<commit_message>
update FPU, control sheet and drawio
</commit_message>
<xml_diff>
--- a/Control.xlsx
+++ b/Control.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Hung\Khoa_Luan\ISS-RV32ICMFA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6FFC3F9-37D3-4720-9414-10674B0D7AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{983697CE-7736-46BF-B58D-410BDE815BBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CF86E8A2-CD57-4282-A2FF-4C2B018B82AC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="134">
   <si>
     <t>instructions</t>
   </si>
@@ -177,9 +177,6 @@
   </si>
   <si>
     <t>xxx</t>
-  </si>
-  <si>
-    <t>PCTargetSrc</t>
   </si>
   <si>
     <t>011</t>
@@ -442,6 +439,18 @@
   </si>
   <si>
     <t>z1</t>
+  </si>
+  <si>
+    <t>addr_addend_sel</t>
+  </si>
+  <si>
+    <t>ResExSel</t>
+  </si>
+  <si>
+    <t>ResPCSel</t>
+  </si>
+  <si>
+    <t>Valid_FPU</t>
   </si>
 </sst>
 </file>
@@ -625,7 +634,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -703,9 +712,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1042,25 +1048,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{690C58A5-C37A-4C5A-8C40-61E7ED87ACAD}">
-  <dimension ref="D3:AJ53"/>
+  <dimension ref="D3:AN54"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="12.77734375" customWidth="1"/>
-    <col min="14" max="14" width="12.44140625" customWidth="1"/>
-    <col min="15" max="15" width="18.109375" customWidth="1"/>
-    <col min="16" max="16" width="10.33203125" customWidth="1"/>
-    <col min="18" max="18" width="8.88671875" customWidth="1"/>
-    <col min="19" max="19" width="9" customWidth="1"/>
-    <col min="20" max="21" width="10.44140625" customWidth="1"/>
-    <col min="22" max="22" width="17.109375" customWidth="1"/>
-    <col min="23" max="23" width="8.88671875" customWidth="1"/>
-    <col min="24" max="24" width="6.109375" customWidth="1"/>
-    <col min="25" max="25" width="17.77734375" customWidth="1"/>
-    <col min="26" max="26" width="14.109375" customWidth="1"/>
-    <col min="27" max="27" width="14.5546875" customWidth="1"/>
+    <col min="14" max="16" width="16.33203125" customWidth="1"/>
+    <col min="17" max="17" width="18.109375" customWidth="1"/>
+    <col min="18" max="18" width="10.33203125" customWidth="1"/>
+    <col min="21" max="21" width="8.88671875" customWidth="1"/>
+    <col min="22" max="22" width="9" customWidth="1"/>
+    <col min="23" max="23" width="10.6640625" customWidth="1"/>
+    <col min="24" max="25" width="10.44140625" customWidth="1"/>
+    <col min="26" max="26" width="17.109375" customWidth="1"/>
+    <col min="27" max="27" width="8.88671875" customWidth="1"/>
+    <col min="28" max="28" width="6.109375" customWidth="1"/>
+    <col min="29" max="29" width="17.77734375" customWidth="1"/>
+    <col min="30" max="30" width="14.109375" customWidth="1"/>
+    <col min="31" max="31" width="14.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="3" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D3" s="17" t="s">
         <v>43</v>
       </c>
@@ -1080,12 +1087,16 @@
       <c r="R3" s="18"/>
       <c r="S3" s="18"/>
       <c r="T3" s="18"/>
-      <c r="U3" s="19"/>
-      <c r="W3" t="s">
+      <c r="U3" s="18"/>
+      <c r="V3" s="18"/>
+      <c r="W3" s="18"/>
+      <c r="X3" s="18"/>
+      <c r="Y3" s="19"/>
+      <c r="AA3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="4" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D4" s="3" t="s">
         <v>0</v>
       </c>
@@ -1117,46 +1128,58 @@
         <v>42</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>47</v>
+        <v>130</v>
       </c>
       <c r="O4" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="R4" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="P4" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="Q4" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="R4" s="3" t="s">
-        <v>72</v>
-      </c>
       <c r="S4" s="3" t="s">
-        <v>92</v>
+        <v>53</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>120</v>
+        <v>56</v>
       </c>
       <c r="U4" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="W4" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="W4" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="X4" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y4" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="AA4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="X4" s="1" t="s">
+      <c r="AB4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="Y4" s="1" t="s">
+      <c r="AC4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="Z4" s="1" t="s">
+      <c r="AD4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="AA4" s="1" t="s">
+      <c r="AE4" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="5" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D5" s="3" t="s">
         <v>1</v>
       </c>
@@ -1193,41 +1216,53 @@
       <c r="O5" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="P5" s="11">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="11">
-        <v>0</v>
-      </c>
-      <c r="R5" s="4" t="s">
+      <c r="P5" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="R5" s="11">
+        <v>0</v>
+      </c>
+      <c r="S5" s="11">
+        <v>0</v>
+      </c>
+      <c r="T5" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="U5" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="S5" s="3">
-        <v>0</v>
-      </c>
-      <c r="T5" s="3">
-        <v>0</v>
-      </c>
-      <c r="U5" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="W5" s="2" t="s">
+      <c r="V5" s="3">
+        <v>0</v>
+      </c>
+      <c r="W5" s="3">
+        <v>0</v>
+      </c>
+      <c r="X5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y5" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="X5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="Y5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="Z5" s="2" t="s">
+      <c r="AB5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="AA5" s="1" t="s">
+      <c r="AE5" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="6" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D6" s="3" t="s">
         <v>2</v>
       </c>
@@ -1264,41 +1299,53 @@
       <c r="O6" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="P6" s="13">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="13">
-        <v>0</v>
-      </c>
-      <c r="R6" s="4" t="s">
+      <c r="P6" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q6" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="R6" s="13">
+        <v>0</v>
+      </c>
+      <c r="S6" s="13">
+        <v>0</v>
+      </c>
+      <c r="T6" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="U6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="S6" s="3">
-        <v>0</v>
-      </c>
-      <c r="T6" s="3">
-        <v>0</v>
-      </c>
-      <c r="U6" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="W6" s="2" t="s">
+      <c r="V6" s="3">
+        <v>0</v>
+      </c>
+      <c r="W6" s="3">
+        <v>0</v>
+      </c>
+      <c r="X6" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="X6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="Y6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="Z6" s="2" t="s">
+      <c r="AB6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="AA6" s="1" t="s">
+      <c r="AE6" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="7" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D7" s="9" t="s">
         <v>3</v>
       </c>
@@ -1332,44 +1379,56 @@
       <c r="N7" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="P7" s="5">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="5">
-        <v>0</v>
-      </c>
-      <c r="R7" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S7" s="3">
-        <v>0</v>
-      </c>
-      <c r="T7" s="3">
-        <v>0</v>
+      <c r="O7" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="P7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="R7" s="5">
+        <v>0</v>
+      </c>
+      <c r="S7" s="5">
+        <v>0</v>
+      </c>
+      <c r="T7" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="U7" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="W7" s="20">
+        <v>46</v>
+      </c>
+      <c r="V7" s="3">
+        <v>0</v>
+      </c>
+      <c r="W7" s="3">
+        <v>0</v>
+      </c>
+      <c r="X7" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA7" s="20">
         <v>10</v>
       </c>
-      <c r="X7" s="2" t="s">
+      <c r="AB7" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="Y7" s="2" t="s">
+      <c r="AC7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="Z7" s="2" t="s">
+      <c r="AD7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="AA7" s="1" t="s">
+      <c r="AE7" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="8" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D8" s="3" t="s">
         <v>44</v>
       </c>
@@ -1406,39 +1465,51 @@
       <c r="O8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="P8" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="3">
-        <v>0</v>
-      </c>
-      <c r="R8" s="3" t="s">
-        <v>46</v>
+      <c r="P8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R8" s="3">
+        <v>0</v>
       </c>
       <c r="S8" s="3">
         <v>0</v>
       </c>
-      <c r="T8" s="3">
-        <v>0</v>
+      <c r="T8" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="U8" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="W8" s="21"/>
-      <c r="X8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="V8" s="3">
+        <v>0</v>
+      </c>
+      <c r="W8" s="3">
+        <v>0</v>
+      </c>
+      <c r="X8" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA8" s="21"/>
+      <c r="AB8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="Y8" s="1">
+      <c r="AC8" s="1">
         <v>11</v>
       </c>
-      <c r="Z8" s="2" t="s">
+      <c r="AD8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="AA8" s="1" t="s">
+      <c r="AE8" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="9" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D9" s="3" t="s">
         <v>36</v>
       </c>
@@ -1472,60 +1543,72 @@
       <c r="N9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="P9" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="3">
-        <v>0</v>
-      </c>
-      <c r="R9" s="3" t="s">
-        <v>46</v>
+      <c r="O9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="P9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R9" s="3">
+        <v>0</v>
       </c>
       <c r="S9" s="3">
         <v>0</v>
       </c>
-      <c r="T9" s="3">
-        <v>0</v>
+      <c r="T9" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="U9" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="W9" s="21"/>
-      <c r="X9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="V9" s="3">
+        <v>0</v>
+      </c>
+      <c r="W9" s="3">
+        <v>0</v>
+      </c>
+      <c r="X9" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA9" s="21"/>
+      <c r="AB9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="Y9" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="Z9" s="1" t="s">
+      <c r="AC9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD9" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AA9" s="1" t="s">
+      <c r="AE9" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AC9" s="1" t="s">
+      <c r="AG9" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AH9" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="AD9" s="1" t="s">
+      <c r="AI9" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="AE9" s="24" t="s">
+      <c r="AJ9" s="24"/>
+      <c r="AK9" s="24"/>
+      <c r="AL9" s="24"/>
+      <c r="AM9" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AF9" s="24"/>
-      <c r="AG9" s="24"/>
-      <c r="AH9" s="24"/>
-      <c r="AI9" s="1" t="s">
+      <c r="AN9" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="AJ9" s="1" t="s">
-        <v>77</v>
-      </c>
     </row>
-    <row r="10" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="10" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D10" s="3" t="s">
         <v>41</v>
       </c>
@@ -1536,7 +1619,7 @@
         <v>1</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>16</v>
@@ -1563,58 +1646,70 @@
         <v>15</v>
       </c>
       <c r="P10" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="3">
-        <v>0</v>
-      </c>
-      <c r="R10" s="3" t="s">
-        <v>46</v>
+        <v>1</v>
+      </c>
+      <c r="Q10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R10" s="3">
+        <v>0</v>
       </c>
       <c r="S10" s="3">
         <v>0</v>
       </c>
-      <c r="T10" s="3">
-        <v>0</v>
+      <c r="T10" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="U10" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="W10" s="21"/>
-      <c r="X10" s="1">
+        <v>46</v>
+      </c>
+      <c r="V10" s="3">
+        <v>0</v>
+      </c>
+      <c r="W10" s="3">
+        <v>0</v>
+      </c>
+      <c r="X10" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA10" s="21"/>
+      <c r="AB10" s="1">
         <v>110</v>
       </c>
-      <c r="Y10" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="Z10" s="1" t="s">
+      <c r="AC10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD10" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AA10" s="1" t="s">
+      <c r="AE10" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AC10" s="14"/>
-      <c r="AD10" s="14"/>
-      <c r="AE10" s="14"/>
-      <c r="AF10" s="1" t="s">
+      <c r="AG10" s="14"/>
+      <c r="AH10" s="14"/>
+      <c r="AI10" s="14"/>
+      <c r="AJ10" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AK10" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="AG10" s="1" t="s">
+      <c r="AL10" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="AH10" s="1" t="s">
+      <c r="AM10" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AI10" s="1" t="s">
+      <c r="AN10" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="AJ10" s="1" t="s">
-        <v>77</v>
-      </c>
     </row>
-    <row r="11" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="11" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D11" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E11" s="4">
         <v>1100111</v>
@@ -1623,7 +1718,7 @@
         <v>1</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>16</v>
@@ -1650,43 +1745,55 @@
         <v>15</v>
       </c>
       <c r="P11" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="3">
-        <v>0</v>
-      </c>
-      <c r="R11" s="3" t="s">
-        <v>46</v>
+        <v>1</v>
+      </c>
+      <c r="Q11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R11" s="3">
+        <v>0</v>
       </c>
       <c r="S11" s="3">
         <v>0</v>
       </c>
-      <c r="T11" s="3">
-        <v>0</v>
+      <c r="T11" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="U11" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="W11" s="22"/>
-      <c r="X11" s="1">
+        <v>46</v>
+      </c>
+      <c r="V11" s="3">
+        <v>0</v>
+      </c>
+      <c r="W11" s="3">
+        <v>0</v>
+      </c>
+      <c r="X11" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA11" s="22"/>
+      <c r="AB11" s="1">
         <v>111</v>
       </c>
-      <c r="Y11" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="Z11" s="1" t="s">
+      <c r="AC11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD11" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AA11" s="1" t="s">
+      <c r="AE11" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="12" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D12" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F12" s="3">
         <v>1</v>
@@ -1701,7 +1808,7 @@
         <v>0</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="K12" s="3">
         <v>0</v>
@@ -1718,31 +1825,43 @@
       <c r="O12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="P12" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="3">
-        <v>0</v>
-      </c>
-      <c r="R12" s="3" t="s">
-        <v>46</v>
+      <c r="P12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R12" s="3">
+        <v>0</v>
       </c>
       <c r="S12" s="3">
         <v>0</v>
       </c>
-      <c r="T12" s="3">
-        <v>0</v>
+      <c r="T12" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="U12" s="3" t="s">
-        <v>123</v>
+        <v>46</v>
+      </c>
+      <c r="V12" s="3">
+        <v>0</v>
+      </c>
+      <c r="W12" s="3">
+        <v>0</v>
+      </c>
+      <c r="X12" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="3" t="s">
+        <v>122</v>
       </c>
     </row>
-    <row r="13" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="13" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D13" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F13" s="3">
         <v>1</v>
@@ -1756,8 +1875,8 @@
       <c r="I13" s="3">
         <v>0</v>
       </c>
-      <c r="J13" s="3">
-        <v>100</v>
+      <c r="J13" s="4" t="s">
+        <v>26</v>
       </c>
       <c r="K13" s="3">
         <v>0</v>
@@ -1768,8 +1887,8 @@
       <c r="M13" s="3">
         <v>0</v>
       </c>
-      <c r="N13" s="3" t="s">
-        <v>16</v>
+      <c r="N13" s="3">
+        <v>0</v>
       </c>
       <c r="O13" s="3" t="s">
         <v>15</v>
@@ -1777,25 +1896,37 @@
       <c r="P13" s="3">
         <v>0</v>
       </c>
-      <c r="Q13" s="3">
-        <v>0</v>
-      </c>
-      <c r="R13" s="3" t="s">
-        <v>46</v>
+      <c r="Q13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R13" s="3">
+        <v>0</v>
       </c>
       <c r="S13" s="3">
         <v>0</v>
       </c>
-      <c r="T13" s="3">
-        <v>0</v>
+      <c r="T13" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="U13" s="3" t="s">
-        <v>123</v>
+        <v>46</v>
+      </c>
+      <c r="V13" s="3">
+        <v>0</v>
+      </c>
+      <c r="W13" s="3">
+        <v>0</v>
+      </c>
+      <c r="X13" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="3" t="s">
+        <v>122</v>
       </c>
     </row>
-    <row r="14" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="14" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D14" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>39</v>
@@ -1812,7 +1943,9 @@
       <c r="I14" s="5">
         <v>0</v>
       </c>
-      <c r="J14" s="5"/>
+      <c r="J14" s="6" t="s">
+        <v>25</v>
+      </c>
       <c r="K14" s="5">
         <v>0</v>
       </c>
@@ -1822,32 +1955,46 @@
       <c r="M14" s="5">
         <v>0</v>
       </c>
-      <c r="N14" s="5"/>
+      <c r="N14" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="O14" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="P14" s="5">
-        <v>1</v>
+        <v>14</v>
+      </c>
+      <c r="P14" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="Q14" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="R14" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S14" s="3">
-        <v>0</v>
-      </c>
-      <c r="T14" s="3">
+      <c r="R14" s="5">
+        <v>1</v>
+      </c>
+      <c r="S14" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="T14" s="6">
         <v>0</v>
       </c>
       <c r="U14" s="3" t="s">
-        <v>123</v>
+        <v>46</v>
+      </c>
+      <c r="V14" s="3">
+        <v>0</v>
+      </c>
+      <c r="W14" s="3">
+        <v>0</v>
+      </c>
+      <c r="X14" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="3" t="s">
+        <v>122</v>
       </c>
     </row>
-    <row r="15" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="15" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D15" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>39</v>
@@ -1864,7 +2011,9 @@
       <c r="I15" s="5">
         <v>0</v>
       </c>
-      <c r="J15" s="5"/>
+      <c r="J15" s="6" t="s">
+        <v>25</v>
+      </c>
       <c r="K15" s="5">
         <v>0</v>
       </c>
@@ -1874,32 +2023,46 @@
       <c r="M15" s="5">
         <v>0</v>
       </c>
-      <c r="N15" s="5"/>
+      <c r="N15" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="O15" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="P15" s="5">
-        <v>1</v>
+      <c r="P15" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="Q15" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="R15" s="5">
+        <v>1</v>
+      </c>
+      <c r="S15" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="R15" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S15" s="3">
-        <v>0</v>
-      </c>
-      <c r="T15" s="3">
-        <v>0</v>
+      <c r="T15" s="6">
+        <v>1</v>
       </c>
       <c r="U15" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V15" s="3">
+        <v>0</v>
+      </c>
+      <c r="W15" s="3">
+        <v>0</v>
+      </c>
+      <c r="X15" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="16" spans="4:40" x14ac:dyDescent="0.3">
+      <c r="D16" s="3" t="s">
         <v>123</v>
-      </c>
-    </row>
-    <row r="16" spans="4:36" x14ac:dyDescent="0.3">
-      <c r="D16" s="3" t="s">
-        <v>124</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>39</v>
@@ -1916,7 +2079,9 @@
       <c r="I16" s="5">
         <v>0</v>
       </c>
-      <c r="J16" s="5"/>
+      <c r="J16" s="6" t="s">
+        <v>25</v>
+      </c>
       <c r="K16" s="5">
         <v>0</v>
       </c>
@@ -1926,32 +2091,46 @@
       <c r="M16" s="5">
         <v>0</v>
       </c>
-      <c r="N16" s="5"/>
-      <c r="O16" s="5">
+      <c r="N16" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="O16" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="P16" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q16" s="5">
         <v>11</v>
       </c>
-      <c r="P16" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q16" s="6" t="s">
+      <c r="R16" s="5">
+        <v>1</v>
+      </c>
+      <c r="S16" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="R16" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S16" s="3">
-        <v>0</v>
-      </c>
-      <c r="T16" s="3">
-        <v>0</v>
+      <c r="T16" s="6">
+        <v>1</v>
       </c>
       <c r="U16" s="3" t="s">
-        <v>123</v>
+        <v>46</v>
+      </c>
+      <c r="V16" s="3">
+        <v>0</v>
+      </c>
+      <c r="W16" s="3">
+        <v>0</v>
+      </c>
+      <c r="X16" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="3" t="s">
+        <v>122</v>
       </c>
     </row>
-    <row r="17" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="17" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D17" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>39</v>
@@ -1968,7 +2147,9 @@
       <c r="I17" s="5">
         <v>0</v>
       </c>
-      <c r="J17" s="5"/>
+      <c r="J17" s="6" t="s">
+        <v>25</v>
+      </c>
       <c r="K17" s="5">
         <v>0</v>
       </c>
@@ -1978,32 +2159,46 @@
       <c r="M17" s="5">
         <v>0</v>
       </c>
-      <c r="N17" s="5"/>
-      <c r="O17" s="5">
-        <v>0</v>
-      </c>
-      <c r="P17" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q17" s="6" t="s">
+      <c r="N17" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="O17" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="P17" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q17" s="5">
+        <v>0</v>
+      </c>
+      <c r="R17" s="5">
+        <v>1</v>
+      </c>
+      <c r="S17" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="R17" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S17" s="3">
-        <v>0</v>
-      </c>
-      <c r="T17" s="3">
-        <v>0</v>
+      <c r="T17" s="6">
+        <v>1</v>
       </c>
       <c r="U17" s="3" t="s">
-        <v>123</v>
+        <v>46</v>
+      </c>
+      <c r="V17" s="3">
+        <v>0</v>
+      </c>
+      <c r="W17" s="3">
+        <v>0</v>
+      </c>
+      <c r="X17" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y17" s="3" t="s">
+        <v>122</v>
       </c>
     </row>
-    <row r="18" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="18" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D18" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>39</v>
@@ -2020,7 +2215,9 @@
       <c r="I18" s="5">
         <v>0</v>
       </c>
-      <c r="J18" s="5"/>
+      <c r="J18" s="6" t="s">
+        <v>25</v>
+      </c>
       <c r="K18" s="5">
         <v>0</v>
       </c>
@@ -2030,32 +2227,46 @@
       <c r="M18" s="5">
         <v>0</v>
       </c>
-      <c r="N18" s="5"/>
-      <c r="O18" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="P18" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q18" s="6" t="s">
+      <c r="N18" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="O18" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="R18" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S18" s="3">
-        <v>0</v>
-      </c>
-      <c r="T18" s="3">
-        <v>0</v>
+      <c r="P18" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q18" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="R18" s="5">
+        <v>1</v>
+      </c>
+      <c r="S18" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="T18" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="U18" s="3" t="s">
-        <v>123</v>
+        <v>46</v>
+      </c>
+      <c r="V18" s="3">
+        <v>0</v>
+      </c>
+      <c r="W18" s="3">
+        <v>0</v>
+      </c>
+      <c r="X18" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="3" t="s">
+        <v>122</v>
       </c>
     </row>
-    <row r="19" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="19" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D19" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>39</v>
@@ -2072,7 +2283,9 @@
       <c r="I19" s="5">
         <v>0</v>
       </c>
-      <c r="J19" s="5"/>
+      <c r="J19" s="6" t="s">
+        <v>25</v>
+      </c>
       <c r="K19" s="5">
         <v>0</v>
       </c>
@@ -2082,32 +2295,46 @@
       <c r="M19" s="5">
         <v>0</v>
       </c>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="P19" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q19" s="6" t="s">
+      <c r="N19" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="O19" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="R19" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S19" s="3">
-        <v>0</v>
-      </c>
-      <c r="T19" s="3">
-        <v>0</v>
+      <c r="P19" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q19" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="R19" s="5">
+        <v>1</v>
+      </c>
+      <c r="S19" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="T19" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="U19" s="3" t="s">
-        <v>123</v>
+        <v>46</v>
+      </c>
+      <c r="V19" s="3">
+        <v>0</v>
+      </c>
+      <c r="W19" s="3">
+        <v>0</v>
+      </c>
+      <c r="X19" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="3" t="s">
+        <v>122</v>
       </c>
     </row>
-    <row r="20" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="20" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D20" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>39</v>
@@ -2124,7 +2351,9 @@
       <c r="I20" s="5">
         <v>0</v>
       </c>
-      <c r="J20" s="5"/>
+      <c r="J20" s="6" t="s">
+        <v>25</v>
+      </c>
       <c r="K20" s="5">
         <v>0</v>
       </c>
@@ -2134,32 +2363,46 @@
       <c r="M20" s="5">
         <v>0</v>
       </c>
-      <c r="N20" s="5"/>
-      <c r="O20" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="P20" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q20" s="5">
+      <c r="N20" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="O20" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="P20" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q20" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="R20" s="5">
+        <v>1</v>
+      </c>
+      <c r="S20" s="5">
         <v>10</v>
       </c>
-      <c r="R20" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S20" s="3">
-        <v>0</v>
-      </c>
-      <c r="T20" s="3">
-        <v>0</v>
+      <c r="T20" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="U20" s="3" t="s">
-        <v>123</v>
+        <v>46</v>
+      </c>
+      <c r="V20" s="3">
+        <v>0</v>
+      </c>
+      <c r="W20" s="3">
+        <v>0</v>
+      </c>
+      <c r="X20" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y20" s="3" t="s">
+        <v>122</v>
       </c>
     </row>
-    <row r="21" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="21" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D21" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>39</v>
@@ -2176,8 +2419,8 @@
       <c r="I21" s="5">
         <v>0</v>
       </c>
-      <c r="J21" s="5">
-        <v>101</v>
+      <c r="J21" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="K21" s="5">
         <v>0</v>
@@ -2191,31 +2434,43 @@
       <c r="N21" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="O21" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="P21" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q21" s="5">
+      <c r="O21" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="P21" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q21" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="R21" s="5">
+        <v>1</v>
+      </c>
+      <c r="S21" s="5">
         <v>10</v>
       </c>
-      <c r="R21" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S21" s="3">
-        <v>0</v>
-      </c>
-      <c r="T21" s="3">
-        <v>0</v>
+      <c r="T21" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="U21" s="3" t="s">
-        <v>123</v>
+        <v>46</v>
+      </c>
+      <c r="V21" s="3">
+        <v>0</v>
+      </c>
+      <c r="W21" s="3">
+        <v>0</v>
+      </c>
+      <c r="X21" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y21" s="3" t="s">
+        <v>122</v>
       </c>
     </row>
-    <row r="22" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="22" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D22" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>37</v>
@@ -2250,45 +2505,57 @@
       <c r="O22" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="P22" s="11">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="11">
-        <v>0</v>
-      </c>
-      <c r="R22" s="4" t="s">
+      <c r="P22" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q22" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="R22" s="11">
+        <v>0</v>
+      </c>
+      <c r="S22" s="11">
+        <v>0</v>
+      </c>
+      <c r="T22" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="U22" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="S22" s="3">
-        <v>0</v>
-      </c>
-      <c r="T22" s="3">
-        <v>0</v>
-      </c>
-      <c r="U22" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="W22" t="s">
-        <v>55</v>
-      </c>
-      <c r="AC22" t="s">
-        <v>78</v>
-      </c>
-      <c r="AD22" s="25" t="s">
-        <v>82</v>
-      </c>
-      <c r="AE22" s="25"/>
-      <c r="AF22" s="25"/>
-      <c r="AG22" s="25" t="s">
-        <v>83</v>
-      </c>
-      <c r="AH22" s="25"/>
+      <c r="V22" s="3">
+        <v>0</v>
+      </c>
+      <c r="W22" s="3">
+        <v>0</v>
+      </c>
+      <c r="X22" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y22" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>54</v>
+      </c>
+      <c r="AG22" t="s">
+        <v>77</v>
+      </c>
+      <c r="AH22" s="25" t="s">
+        <v>81</v>
+      </c>
       <c r="AI22" s="25"/>
       <c r="AJ22" s="25"/>
+      <c r="AK22" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="AL22" s="25"/>
+      <c r="AM22" s="25"/>
+      <c r="AN22" s="25"/>
     </row>
-    <row r="23" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="23" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D23" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>37</v>
@@ -2323,57 +2590,69 @@
       <c r="O23" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="P23" s="11">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="11">
-        <v>0</v>
-      </c>
-      <c r="R23" s="4" t="s">
+      <c r="P23" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q23" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="R23" s="11">
+        <v>0</v>
+      </c>
+      <c r="S23" s="11">
+        <v>0</v>
+      </c>
+      <c r="T23" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="U23" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="S23" s="3">
-        <v>0</v>
-      </c>
-      <c r="T23" s="3">
-        <v>0</v>
-      </c>
-      <c r="U23" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="W23" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="X23" s="1" t="s">
+      <c r="V23" s="3">
+        <v>0</v>
+      </c>
+      <c r="W23" s="3">
+        <v>0</v>
+      </c>
+      <c r="X23" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y23" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA23" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB23" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="Y23" s="1" t="s">
+      <c r="AC23" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AD23" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="Z23" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="AA23" s="1" t="s">
+      <c r="AE23" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="AC23" s="1" t="s">
+      <c r="AG23" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="AH23" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="AD23" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="AE23" s="24"/>
-      <c r="AF23" s="24"/>
-      <c r="AG23" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="AH23" s="24"/>
       <c r="AI23" s="24"/>
       <c r="AJ23" s="24"/>
+      <c r="AK23" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="AL23" s="24"/>
+      <c r="AM23" s="24"/>
+      <c r="AN23" s="24"/>
     </row>
-    <row r="24" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="24" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D24" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>37</v>
@@ -2408,43 +2687,55 @@
       <c r="O24" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="P24" s="11">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="11">
-        <v>0</v>
-      </c>
-      <c r="R24" s="3">
+      <c r="P24" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q24" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="R24" s="11">
+        <v>0</v>
+      </c>
+      <c r="S24" s="11">
+        <v>0</v>
+      </c>
+      <c r="T24" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="U24" s="3">
         <v>101</v>
       </c>
-      <c r="S24" s="3">
-        <v>0</v>
-      </c>
-      <c r="T24" s="3">
-        <v>0</v>
-      </c>
-      <c r="U24" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="W24" s="2">
-        <v>0</v>
-      </c>
-      <c r="X24" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="Y24" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Z24" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AA24" s="1" t="s">
+      <c r="V24" s="3">
+        <v>0</v>
+      </c>
+      <c r="W24" s="3">
+        <v>0</v>
+      </c>
+      <c r="X24" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y24" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA24" s="2">
+        <v>0</v>
+      </c>
+      <c r="AB24" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC24" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE24" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="25" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D25" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>37</v>
@@ -2479,56 +2770,68 @@
       <c r="O25" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="P25" s="11">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="11">
-        <v>0</v>
-      </c>
-      <c r="R25" s="3">
+      <c r="P25" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q25" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="R25" s="11">
+        <v>0</v>
+      </c>
+      <c r="S25" s="11">
+        <v>0</v>
+      </c>
+      <c r="T25" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="U25" s="3">
         <v>110</v>
       </c>
-      <c r="S25" s="3">
-        <v>0</v>
-      </c>
-      <c r="T25" s="3">
-        <v>0</v>
-      </c>
-      <c r="U25" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="W25" s="23">
-        <v>1</v>
-      </c>
-      <c r="X25" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y25" s="2" t="s">
+      <c r="V25" s="3">
+        <v>0</v>
+      </c>
+      <c r="W25" s="3">
+        <v>0</v>
+      </c>
+      <c r="X25" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y25" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA25" s="23">
+        <v>1</v>
+      </c>
+      <c r="AB25" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC25" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="Z25" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA25" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="AC25" s="3" t="s">
+      <c r="AD25" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE25" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AG25" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="AH25" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="AD25" s="3" t="s">
+      <c r="AI25" s="3"/>
+      <c r="AJ25" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="AE25" s="3"/>
-      <c r="AF25" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="AG25" s="26"/>
-      <c r="AH25" s="26"/>
-      <c r="AI25" s="26"/>
+      <c r="AK25" s="26"/>
+      <c r="AL25" s="26"/>
+      <c r="AM25" s="26"/>
     </row>
-    <row r="26" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="26" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D26" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E26" s="8" t="s">
         <v>38</v>
@@ -2563,54 +2866,66 @@
       <c r="O26" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="P26" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="15">
-        <v>0</v>
-      </c>
-      <c r="R26" s="4" t="s">
+      <c r="P26" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q26" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="R26" s="15">
+        <v>0</v>
+      </c>
+      <c r="S26" s="15">
+        <v>0</v>
+      </c>
+      <c r="T26" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="U26" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="S26" s="3">
-        <v>0</v>
-      </c>
-      <c r="T26" s="3">
-        <v>0</v>
-      </c>
-      <c r="U26" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="W26" s="23"/>
-      <c r="X26" s="2">
-        <v>1</v>
-      </c>
-      <c r="Y26" s="2" t="s">
+      <c r="V26" s="3">
+        <v>0</v>
+      </c>
+      <c r="W26" s="3">
+        <v>0</v>
+      </c>
+      <c r="X26" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y26" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA26" s="23"/>
+      <c r="AB26" s="2">
+        <v>1</v>
+      </c>
+      <c r="AC26" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="Z26" s="2">
-        <v>1</v>
-      </c>
-      <c r="AA26" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="AC26" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD26" s="26">
+      <c r="AD26" s="2">
+        <v>1</v>
+      </c>
+      <c r="AE26" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AG26" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH26" s="26">
         <v>-127</v>
       </c>
-      <c r="AE26" s="26"/>
-      <c r="AF26" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="AG26" s="26"/>
-      <c r="AH26" s="26"/>
       <c r="AI26" s="26"/>
+      <c r="AJ26" s="26" t="s">
+        <v>88</v>
+      </c>
+      <c r="AK26" s="26"/>
+      <c r="AL26" s="26"/>
+      <c r="AM26" s="26"/>
     </row>
-    <row r="27" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="27" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D27" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E27" s="8" t="s">
         <v>38</v>
@@ -2645,57 +2960,69 @@
       <c r="O27" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="P27" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="15">
-        <v>0</v>
-      </c>
-      <c r="R27" s="4" t="s">
+      <c r="P27" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q27" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="R27" s="15">
+        <v>0</v>
+      </c>
+      <c r="S27" s="15">
+        <v>0</v>
+      </c>
+      <c r="T27" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="U27" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="S27" s="3">
-        <v>0</v>
-      </c>
-      <c r="T27" s="3">
-        <v>0</v>
-      </c>
-      <c r="U27" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="W27" s="23"/>
-      <c r="X27" s="2">
+      <c r="V27" s="3">
+        <v>0</v>
+      </c>
+      <c r="W27" s="3">
+        <v>0</v>
+      </c>
+      <c r="X27" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y27" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA27" s="23"/>
+      <c r="AB27" s="2">
         <v>2</v>
       </c>
-      <c r="Y27" s="1">
+      <c r="AC27" s="1">
         <v>11</v>
       </c>
-      <c r="Z27" s="2">
-        <v>1</v>
-      </c>
-      <c r="AA27" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="AC27" s="3" t="s">
+      <c r="AD27" s="2">
+        <v>1</v>
+      </c>
+      <c r="AE27" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="AG27" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="AH27" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="AD27" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="AE27" s="23"/>
-      <c r="AF27" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="AG27" s="26"/>
-      <c r="AH27" s="26"/>
-      <c r="AI27" s="26"/>
+      <c r="AI27" s="23"/>
+      <c r="AJ27" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="AK27" s="26"/>
+      <c r="AL27" s="26"/>
+      <c r="AM27" s="26"/>
     </row>
-    <row r="28" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="28" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D28" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F28" s="3">
         <v>0</v>
@@ -2710,7 +3037,7 @@
         <v>0</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="K28" s="3">
         <v>0</v>
@@ -2724,60 +3051,72 @@
       <c r="N28" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O28" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P28" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="3">
-        <v>0</v>
-      </c>
-      <c r="R28" s="4" t="s">
+      <c r="O28" s="3">
+        <v>10</v>
+      </c>
+      <c r="P28" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q28" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R28" s="3">
+        <v>0</v>
+      </c>
+      <c r="S28" s="3">
+        <v>0</v>
+      </c>
+      <c r="T28" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U28" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="S28" s="3">
-        <v>1</v>
-      </c>
-      <c r="T28" s="3">
-        <v>1</v>
-      </c>
-      <c r="U28" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="W28" s="23"/>
-      <c r="X28" s="2">
+      <c r="V28" s="3">
+        <v>1</v>
+      </c>
+      <c r="W28" s="3">
+        <v>1</v>
+      </c>
+      <c r="X28" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y28" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA28" s="23"/>
+      <c r="AB28" s="2">
         <v>3</v>
       </c>
-      <c r="Y28" s="2" t="s">
+      <c r="AC28" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="Z28" s="1">
-        <v>1</v>
-      </c>
-      <c r="AA28" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC28" s="3">
+      <c r="AD28" s="1">
+        <v>1</v>
+      </c>
+      <c r="AE28" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG28" s="3">
         <v>255</v>
       </c>
-      <c r="AD28" s="26">
+      <c r="AH28" s="26">
         <v>128</v>
       </c>
-      <c r="AE28" s="26"/>
-      <c r="AF28" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="AG28" s="26"/>
-      <c r="AH28" s="26"/>
       <c r="AI28" s="26"/>
+      <c r="AJ28" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="AK28" s="26"/>
+      <c r="AL28" s="26"/>
+      <c r="AM28" s="26"/>
     </row>
-    <row r="29" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="29" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D29" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F29" s="3">
         <v>0</v>
@@ -2791,8 +3130,8 @@
       <c r="I29" s="3">
         <v>1</v>
       </c>
-      <c r="J29" s="3" t="s">
-        <v>46</v>
+      <c r="J29" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K29" s="3">
         <v>0</v>
@@ -2806,44 +3145,56 @@
       <c r="N29" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O29" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P29" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q29" s="3">
-        <v>0</v>
-      </c>
-      <c r="R29" s="4" t="s">
+      <c r="O29" s="3">
+        <v>10</v>
+      </c>
+      <c r="P29" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q29" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R29" s="3">
+        <v>0</v>
+      </c>
+      <c r="S29" s="3">
+        <v>0</v>
+      </c>
+      <c r="T29" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U29" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="S29" s="3">
-        <v>0</v>
-      </c>
-      <c r="T29" s="3">
-        <v>1</v>
-      </c>
-      <c r="U29" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="W29" s="23"/>
-      <c r="X29" s="1">
+      <c r="V29" s="3">
+        <v>0</v>
+      </c>
+      <c r="W29" s="3">
+        <v>1</v>
+      </c>
+      <c r="X29" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y29" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA29" s="23"/>
+      <c r="AB29" s="1">
         <v>4</v>
       </c>
-      <c r="Y29" s="2" t="s">
+      <c r="AC29" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="Z29" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="AA29" s="1" t="s">
-        <v>62</v>
+      <c r="AD29" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE29" s="1" t="s">
+        <v>61</v>
       </c>
     </row>
-    <row r="30" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="30" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D30" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E30" s="3">
         <v>1000011</v>
@@ -2860,8 +3211,8 @@
       <c r="I30" s="3">
         <v>0</v>
       </c>
-      <c r="J30" s="3">
-        <v>110</v>
+      <c r="J30" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K30" s="3">
         <v>0</v>
@@ -2875,44 +3226,56 @@
       <c r="N30" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O30" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P30" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="3">
-        <v>0</v>
-      </c>
-      <c r="R30" s="3" t="s">
-        <v>46</v>
+      <c r="O30" s="3">
+        <v>10</v>
+      </c>
+      <c r="P30" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q30" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R30" s="3">
+        <v>0</v>
       </c>
       <c r="S30" s="3">
-        <v>1</v>
-      </c>
-      <c r="T30" s="3">
-        <v>1</v>
-      </c>
-      <c r="U30" s="3">
+        <v>0</v>
+      </c>
+      <c r="T30" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U30" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V30" s="3">
+        <v>1</v>
+      </c>
+      <c r="W30" s="3">
+        <v>1</v>
+      </c>
+      <c r="X30" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y30" s="3">
         <v>11</v>
       </c>
-      <c r="W30" s="23"/>
-      <c r="X30" s="1">
+      <c r="AA30" s="23"/>
+      <c r="AB30" s="1">
         <v>5</v>
       </c>
-      <c r="Y30" s="2" t="s">
+      <c r="AC30" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="Z30" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="AA30" s="1" t="s">
-        <v>63</v>
+      <c r="AD30" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE30" s="1" t="s">
+        <v>62</v>
       </c>
     </row>
-    <row r="31" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="31" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D31" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E31" s="3">
         <v>1000111</v>
@@ -2929,8 +3292,8 @@
       <c r="I31" s="3">
         <v>0</v>
       </c>
-      <c r="J31" s="3">
-        <v>110</v>
+      <c r="J31" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K31" s="3">
         <v>0</v>
@@ -2944,44 +3307,56 @@
       <c r="N31" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O31" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P31" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q31" s="3">
-        <v>0</v>
-      </c>
-      <c r="R31" s="3" t="s">
-        <v>46</v>
+      <c r="O31" s="3">
+        <v>10</v>
+      </c>
+      <c r="P31" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q31" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R31" s="3">
+        <v>0</v>
       </c>
       <c r="S31" s="3">
-        <v>1</v>
-      </c>
-      <c r="T31" s="3">
-        <v>1</v>
-      </c>
-      <c r="U31" s="3">
+        <v>0</v>
+      </c>
+      <c r="T31" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U31" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V31" s="3">
+        <v>1</v>
+      </c>
+      <c r="W31" s="3">
+        <v>1</v>
+      </c>
+      <c r="X31" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y31" s="3">
         <v>12</v>
       </c>
-      <c r="W31" s="23"/>
-      <c r="X31" s="1">
+      <c r="AA31" s="23"/>
+      <c r="AB31" s="1">
         <v>6</v>
       </c>
-      <c r="Y31" s="2" t="s">
+      <c r="AC31" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="Z31" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="AA31" s="1" t="s">
-        <v>64</v>
+      <c r="AD31" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE31" s="1" t="s">
+        <v>63</v>
       </c>
     </row>
-    <row r="32" spans="4:36" x14ac:dyDescent="0.3">
+    <row r="32" spans="4:40" x14ac:dyDescent="0.3">
       <c r="D32" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E32" s="3">
         <v>1001111</v>
@@ -2998,8 +3373,8 @@
       <c r="I32" s="3">
         <v>0</v>
       </c>
-      <c r="J32" s="3">
-        <v>110</v>
+      <c r="J32" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K32" s="3">
         <v>0</v>
@@ -3013,44 +3388,56 @@
       <c r="N32" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O32" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P32" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q32" s="3">
-        <v>0</v>
-      </c>
-      <c r="R32" s="3" t="s">
-        <v>46</v>
+      <c r="O32" s="3">
+        <v>10</v>
+      </c>
+      <c r="P32" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q32" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R32" s="3">
+        <v>0</v>
       </c>
       <c r="S32" s="3">
-        <v>1</v>
-      </c>
-      <c r="T32" s="3">
-        <v>1</v>
-      </c>
-      <c r="U32" s="3">
+        <v>0</v>
+      </c>
+      <c r="T32" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U32" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V32" s="3">
+        <v>1</v>
+      </c>
+      <c r="W32" s="3">
+        <v>1</v>
+      </c>
+      <c r="X32" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y32" s="3">
         <v>13</v>
       </c>
-      <c r="W32" s="23"/>
-      <c r="X32" s="1">
+      <c r="AA32" s="23"/>
+      <c r="AB32" s="1">
         <v>7</v>
       </c>
-      <c r="Y32" s="2" t="s">
+      <c r="AC32" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="Z32" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="AA32" s="1" t="s">
-        <v>65</v>
+      <c r="AD32" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE32" s="1" t="s">
+        <v>64</v>
       </c>
     </row>
-    <row r="33" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="33" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D33" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E33" s="3">
         <v>1001011</v>
@@ -3067,8 +3454,8 @@
       <c r="I33" s="3">
         <v>0</v>
       </c>
-      <c r="J33" s="3">
-        <v>110</v>
+      <c r="J33" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K33" s="3">
         <v>0</v>
@@ -3082,31 +3469,43 @@
       <c r="N33" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O33" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P33" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q33" s="3">
-        <v>0</v>
-      </c>
-      <c r="R33" s="3" t="s">
-        <v>46</v>
+      <c r="O33" s="3">
+        <v>10</v>
+      </c>
+      <c r="P33" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q33" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R33" s="3">
+        <v>0</v>
       </c>
       <c r="S33" s="3">
-        <v>1</v>
-      </c>
-      <c r="T33" s="3">
-        <v>1</v>
-      </c>
-      <c r="U33" s="3">
+        <v>0</v>
+      </c>
+      <c r="T33" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U33" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V33" s="3">
+        <v>1</v>
+      </c>
+      <c r="W33" s="3">
+        <v>1</v>
+      </c>
+      <c r="X33" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y33" s="3">
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="34" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D34" s="16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E34" s="3">
         <v>1010011</v>
@@ -3123,8 +3522,8 @@
       <c r="I34" s="3">
         <v>0</v>
       </c>
-      <c r="J34" s="3">
-        <v>110</v>
+      <c r="J34" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K34" s="3">
         <v>0</v>
@@ -3138,31 +3537,43 @@
       <c r="N34" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O34" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P34" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q34" s="3">
-        <v>0</v>
-      </c>
-      <c r="R34" s="3" t="s">
-        <v>46</v>
+      <c r="O34" s="3">
+        <v>10</v>
+      </c>
+      <c r="P34" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q34" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R34" s="3">
+        <v>0</v>
       </c>
       <c r="S34" s="3">
-        <v>1</v>
-      </c>
-      <c r="T34" s="3">
-        <v>1</v>
-      </c>
-      <c r="U34" s="3">
+        <v>0</v>
+      </c>
+      <c r="T34" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U34" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V34" s="3">
+        <v>1</v>
+      </c>
+      <c r="W34" s="3">
+        <v>1</v>
+      </c>
+      <c r="X34" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y34" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="35" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D35" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E35" s="3">
         <v>1010011</v>
@@ -3179,8 +3590,8 @@
       <c r="I35" s="3">
         <v>0</v>
       </c>
-      <c r="J35" s="3">
-        <v>110</v>
+      <c r="J35" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K35" s="3">
         <v>0</v>
@@ -3194,31 +3605,43 @@
       <c r="N35" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O35" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P35" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q35" s="3">
-        <v>0</v>
-      </c>
-      <c r="R35" s="3" t="s">
-        <v>46</v>
+      <c r="O35" s="3">
+        <v>10</v>
+      </c>
+      <c r="P35" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q35" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R35" s="3">
+        <v>0</v>
       </c>
       <c r="S35" s="3">
-        <v>1</v>
-      </c>
-      <c r="T35" s="3">
-        <v>1</v>
-      </c>
-      <c r="U35" s="3">
+        <v>0</v>
+      </c>
+      <c r="T35" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U35" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V35" s="3">
+        <v>1</v>
+      </c>
+      <c r="W35" s="3">
+        <v>1</v>
+      </c>
+      <c r="X35" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y35" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="36" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D36" s="16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E36" s="3">
         <v>1010011</v>
@@ -3235,8 +3658,8 @@
       <c r="I36" s="3">
         <v>0</v>
       </c>
-      <c r="J36" s="3">
-        <v>110</v>
+      <c r="J36" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K36" s="3">
         <v>0</v>
@@ -3250,31 +3673,43 @@
       <c r="N36" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O36" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P36" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q36" s="3">
-        <v>0</v>
-      </c>
-      <c r="R36" s="3" t="s">
-        <v>46</v>
+      <c r="O36" s="3">
+        <v>10</v>
+      </c>
+      <c r="P36" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q36" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R36" s="3">
+        <v>0</v>
       </c>
       <c r="S36" s="3">
-        <v>1</v>
-      </c>
-      <c r="T36" s="3">
-        <v>1</v>
-      </c>
-      <c r="U36" s="3">
+        <v>0</v>
+      </c>
+      <c r="T36" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U36" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V36" s="3">
+        <v>1</v>
+      </c>
+      <c r="W36" s="3">
+        <v>1</v>
+      </c>
+      <c r="X36" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y36" s="3">
         <v>17</v>
       </c>
     </row>
-    <row r="37" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="37" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D37" s="16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E37" s="3">
         <v>1010011</v>
@@ -3291,8 +3726,8 @@
       <c r="I37" s="3">
         <v>0</v>
       </c>
-      <c r="J37" s="3">
-        <v>110</v>
+      <c r="J37" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K37" s="3">
         <v>0</v>
@@ -3306,31 +3741,43 @@
       <c r="N37" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O37" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P37" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q37" s="3">
-        <v>0</v>
-      </c>
-      <c r="R37" s="3" t="s">
-        <v>46</v>
+      <c r="O37" s="3">
+        <v>10</v>
+      </c>
+      <c r="P37" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q37" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R37" s="3">
+        <v>0</v>
       </c>
       <c r="S37" s="3">
-        <v>1</v>
-      </c>
-      <c r="T37" s="3">
-        <v>1</v>
-      </c>
-      <c r="U37" s="3">
+        <v>0</v>
+      </c>
+      <c r="T37" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U37" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V37" s="3">
+        <v>1</v>
+      </c>
+      <c r="W37" s="3">
+        <v>1</v>
+      </c>
+      <c r="X37" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y37" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="38" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D38" s="16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E38" s="3">
         <v>1010011</v>
@@ -3347,8 +3794,8 @@
       <c r="I38" s="3">
         <v>0</v>
       </c>
-      <c r="J38" s="3">
-        <v>110</v>
+      <c r="J38" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K38" s="3">
         <v>0</v>
@@ -3362,31 +3809,43 @@
       <c r="N38" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O38" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P38" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q38" s="3">
-        <v>0</v>
-      </c>
-      <c r="R38" s="3" t="s">
-        <v>46</v>
+      <c r="O38" s="3">
+        <v>10</v>
+      </c>
+      <c r="P38" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q38" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R38" s="3">
+        <v>0</v>
       </c>
       <c r="S38" s="3">
-        <v>1</v>
-      </c>
-      <c r="T38" s="3">
-        <v>1</v>
-      </c>
-      <c r="U38" s="3">
+        <v>0</v>
+      </c>
+      <c r="T38" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U38" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V38" s="3">
+        <v>1</v>
+      </c>
+      <c r="W38" s="3">
+        <v>1</v>
+      </c>
+      <c r="X38" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y38" s="3">
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="39" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D39" s="16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E39" s="3">
         <v>1010011</v>
@@ -3403,8 +3862,8 @@
       <c r="I39" s="3">
         <v>0</v>
       </c>
-      <c r="J39" s="3">
-        <v>110</v>
+      <c r="J39" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K39" s="3">
         <v>0</v>
@@ -3418,31 +3877,43 @@
       <c r="N39" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O39" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P39" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q39" s="3">
-        <v>0</v>
-      </c>
-      <c r="R39" s="3" t="s">
-        <v>46</v>
+      <c r="O39" s="3">
+        <v>10</v>
+      </c>
+      <c r="P39" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q39" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R39" s="3">
+        <v>0</v>
       </c>
       <c r="S39" s="3">
-        <v>1</v>
-      </c>
-      <c r="T39" s="3">
-        <v>1</v>
-      </c>
-      <c r="U39" s="3">
+        <v>0</v>
+      </c>
+      <c r="T39" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U39" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V39" s="3">
+        <v>1</v>
+      </c>
+      <c r="W39" s="3">
+        <v>1</v>
+      </c>
+      <c r="X39" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y39" s="3">
         <v>18</v>
       </c>
     </row>
-    <row r="40" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="40" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D40" s="16" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E40" s="3">
         <v>1010011</v>
@@ -3459,8 +3930,8 @@
       <c r="I40" s="3">
         <v>0</v>
       </c>
-      <c r="J40" s="3">
-        <v>110</v>
+      <c r="J40" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K40" s="3">
         <v>0</v>
@@ -3474,31 +3945,43 @@
       <c r="N40" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O40" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P40" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q40" s="3">
-        <v>0</v>
-      </c>
-      <c r="R40" s="3" t="s">
-        <v>46</v>
+      <c r="O40" s="3">
+        <v>10</v>
+      </c>
+      <c r="P40" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q40" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R40" s="3">
+        <v>0</v>
       </c>
       <c r="S40" s="3">
-        <v>1</v>
-      </c>
-      <c r="T40" s="3">
-        <v>1</v>
-      </c>
-      <c r="U40" s="3">
+        <v>0</v>
+      </c>
+      <c r="T40" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U40" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V40" s="3">
+        <v>1</v>
+      </c>
+      <c r="W40" s="3">
+        <v>1</v>
+      </c>
+      <c r="X40" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y40" s="3">
         <v>19</v>
       </c>
     </row>
-    <row r="41" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="41" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D41" s="16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E41" s="3">
         <v>1010011</v>
@@ -3515,8 +3998,8 @@
       <c r="I41" s="3">
         <v>0</v>
       </c>
-      <c r="J41" s="3">
-        <v>110</v>
+      <c r="J41" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K41" s="3">
         <v>0</v>
@@ -3530,31 +4013,43 @@
       <c r="N41" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O41" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P41" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q41" s="3">
-        <v>0</v>
-      </c>
-      <c r="R41" s="3" t="s">
-        <v>46</v>
+      <c r="O41" s="3">
+        <v>10</v>
+      </c>
+      <c r="P41" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q41" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R41" s="3">
+        <v>0</v>
       </c>
       <c r="S41" s="3">
-        <v>1</v>
-      </c>
-      <c r="T41" s="3">
-        <v>1</v>
-      </c>
-      <c r="U41" s="3">
+        <v>0</v>
+      </c>
+      <c r="T41" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U41" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V41" s="3">
+        <v>1</v>
+      </c>
+      <c r="W41" s="3">
+        <v>1</v>
+      </c>
+      <c r="X41" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y41" s="3">
         <v>20</v>
       </c>
     </row>
-    <row r="42" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="42" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D42" s="16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E42" s="3">
         <v>1010011</v>
@@ -3571,8 +4066,8 @@
       <c r="I42" s="3">
         <v>0</v>
       </c>
-      <c r="J42" s="3">
-        <v>110</v>
+      <c r="J42" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K42" s="3">
         <v>0</v>
@@ -3586,31 +4081,43 @@
       <c r="N42" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O42" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P42" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q42" s="3">
-        <v>0</v>
-      </c>
-      <c r="R42" s="3" t="s">
-        <v>46</v>
+      <c r="O42" s="3">
+        <v>10</v>
+      </c>
+      <c r="P42" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q42" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R42" s="3">
+        <v>0</v>
       </c>
       <c r="S42" s="3">
-        <v>1</v>
-      </c>
-      <c r="T42" s="3">
-        <v>1</v>
-      </c>
-      <c r="U42" s="3">
+        <v>0</v>
+      </c>
+      <c r="T42" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U42" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V42" s="3">
+        <v>1</v>
+      </c>
+      <c r="W42" s="3">
+        <v>1</v>
+      </c>
+      <c r="X42" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y42" s="3">
         <v>16</v>
       </c>
     </row>
-    <row r="43" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="43" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D43" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E43" s="3">
         <v>1010011</v>
@@ -3627,8 +4134,8 @@
       <c r="I43" s="3">
         <v>0</v>
       </c>
-      <c r="J43" s="3">
-        <v>110</v>
+      <c r="J43" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K43" s="3">
         <v>0</v>
@@ -3642,31 +4149,43 @@
       <c r="N43" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O43" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P43" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q43" s="3">
-        <v>0</v>
-      </c>
-      <c r="R43" s="3" t="s">
-        <v>46</v>
+      <c r="O43" s="3">
+        <v>10</v>
+      </c>
+      <c r="P43" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q43" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R43" s="3">
+        <v>0</v>
       </c>
       <c r="S43" s="3">
-        <v>1</v>
-      </c>
-      <c r="T43" s="3">
-        <v>1</v>
-      </c>
-      <c r="U43" s="3">
+        <v>0</v>
+      </c>
+      <c r="T43" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U43" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V43" s="3">
+        <v>1</v>
+      </c>
+      <c r="W43" s="3">
+        <v>1</v>
+      </c>
+      <c r="X43" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y43" s="3">
         <v>15</v>
       </c>
     </row>
-    <row r="44" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="44" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D44" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E44" s="3">
         <v>1010011</v>
@@ -3683,8 +4202,8 @@
       <c r="I44" s="3">
         <v>0</v>
       </c>
-      <c r="J44" s="3">
-        <v>110</v>
+      <c r="J44" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K44" s="3">
         <v>0</v>
@@ -3698,31 +4217,43 @@
       <c r="N44" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O44" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P44" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q44" s="3">
-        <v>0</v>
-      </c>
-      <c r="R44" s="3" t="s">
-        <v>46</v>
+      <c r="O44" s="3">
+        <v>10</v>
+      </c>
+      <c r="P44" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q44" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R44" s="3">
+        <v>0</v>
       </c>
       <c r="S44" s="3">
-        <v>1</v>
-      </c>
-      <c r="T44" s="3">
-        <v>1</v>
-      </c>
-      <c r="U44" s="3">
+        <v>0</v>
+      </c>
+      <c r="T44" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U44" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V44" s="3">
+        <v>1</v>
+      </c>
+      <c r="W44" s="3">
+        <v>1</v>
+      </c>
+      <c r="X44" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y44" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="45" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D45" s="16" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E45" s="3">
         <v>1010011</v>
@@ -3739,46 +4270,58 @@
       <c r="I45" s="3">
         <v>0</v>
       </c>
-      <c r="J45" s="3">
+      <c r="J45" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K45" s="3">
+        <v>0</v>
+      </c>
+      <c r="L45" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="M45" s="3">
+        <v>0</v>
+      </c>
+      <c r="N45" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="O45" s="3">
+        <v>10</v>
+      </c>
+      <c r="P45" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q45" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R45" s="3">
+        <v>0</v>
+      </c>
+      <c r="S45" s="3">
+        <v>0</v>
+      </c>
+      <c r="T45" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U45" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V45" s="3">
+        <v>1</v>
+      </c>
+      <c r="W45" s="3">
+        <v>1</v>
+      </c>
+      <c r="X45" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y45" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="46" spans="4:25" x14ac:dyDescent="0.3">
+      <c r="D46" s="16" t="s">
         <v>110</v>
-      </c>
-      <c r="K45" s="3">
-        <v>0</v>
-      </c>
-      <c r="L45" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="M45" s="3">
-        <v>0</v>
-      </c>
-      <c r="N45" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="O45" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P45" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q45" s="3">
-        <v>0</v>
-      </c>
-      <c r="R45" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S45" s="3">
-        <v>1</v>
-      </c>
-      <c r="T45" s="3">
-        <v>1</v>
-      </c>
-      <c r="U45" s="3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="46" spans="4:21" x14ac:dyDescent="0.3">
-      <c r="D46" s="16" t="s">
-        <v>111</v>
       </c>
       <c r="E46" s="3">
         <v>1010011</v>
@@ -3795,8 +4338,8 @@
       <c r="I46" s="3">
         <v>0</v>
       </c>
-      <c r="J46" s="3">
-        <v>110</v>
+      <c r="J46" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K46" s="3">
         <v>0</v>
@@ -3810,31 +4353,43 @@
       <c r="N46" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O46" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P46" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q46" s="3">
-        <v>0</v>
-      </c>
-      <c r="R46" s="3" t="s">
-        <v>46</v>
+      <c r="O46" s="3">
+        <v>10</v>
+      </c>
+      <c r="P46" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q46" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R46" s="3">
+        <v>0</v>
       </c>
       <c r="S46" s="3">
-        <v>1</v>
-      </c>
-      <c r="T46" s="3">
-        <v>1</v>
-      </c>
-      <c r="U46" s="3">
+        <v>0</v>
+      </c>
+      <c r="T46" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U46" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V46" s="3">
+        <v>1</v>
+      </c>
+      <c r="W46" s="3">
+        <v>1</v>
+      </c>
+      <c r="X46" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y46" s="3">
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="47" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D47" s="16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E47" s="3">
         <v>1010011</v>
@@ -3851,8 +4406,8 @@
       <c r="I47" s="3">
         <v>0</v>
       </c>
-      <c r="J47" s="3">
-        <v>110</v>
+      <c r="J47" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K47" s="3">
         <v>0</v>
@@ -3866,37 +4421,49 @@
       <c r="N47" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O47" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P47" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q47" s="3">
-        <v>0</v>
-      </c>
-      <c r="R47" s="3" t="s">
-        <v>46</v>
+      <c r="O47" s="3">
+        <v>10</v>
+      </c>
+      <c r="P47" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q47" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R47" s="3">
+        <v>0</v>
       </c>
       <c r="S47" s="3">
-        <v>1</v>
-      </c>
-      <c r="T47" s="3">
-        <v>1</v>
-      </c>
-      <c r="U47" s="3">
+        <v>0</v>
+      </c>
+      <c r="T47" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U47" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V47" s="3">
+        <v>1</v>
+      </c>
+      <c r="W47" s="3">
+        <v>1</v>
+      </c>
+      <c r="X47" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y47" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="48" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="48" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D48" s="16" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E48" s="3">
         <v>1010011</v>
       </c>
       <c r="F48" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G48" s="3" t="s">
         <v>46</v>
@@ -3907,8 +4474,8 @@
       <c r="I48" s="3">
         <v>0</v>
       </c>
-      <c r="J48" s="3">
-        <v>110</v>
+      <c r="J48" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K48" s="3">
         <v>0</v>
@@ -3922,31 +4489,43 @@
       <c r="N48" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O48" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P48" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q48" s="3">
-        <v>0</v>
-      </c>
-      <c r="R48" s="3" t="s">
-        <v>46</v>
+      <c r="O48" s="3">
+        <v>10</v>
+      </c>
+      <c r="P48" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q48" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R48" s="3">
+        <v>0</v>
       </c>
       <c r="S48" s="3">
-        <v>1</v>
-      </c>
-      <c r="T48" s="3">
-        <v>1</v>
-      </c>
-      <c r="U48" s="3">
+        <v>0</v>
+      </c>
+      <c r="T48" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U48" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V48" s="3">
+        <v>0</v>
+      </c>
+      <c r="W48" s="3">
+        <v>1</v>
+      </c>
+      <c r="X48" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y48" s="3">
         <v>22</v>
       </c>
     </row>
-    <row r="49" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="49" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D49" s="16" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E49" s="3">
         <v>1010011</v>
@@ -3963,8 +4542,8 @@
       <c r="I49" s="3">
         <v>0</v>
       </c>
-      <c r="J49" s="3">
-        <v>110</v>
+      <c r="J49" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K49" s="3">
         <v>0</v>
@@ -3978,31 +4557,43 @@
       <c r="N49" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O49" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P49" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q49" s="3">
-        <v>0</v>
-      </c>
-      <c r="R49" s="3" t="s">
-        <v>46</v>
+      <c r="O49" s="3">
+        <v>10</v>
+      </c>
+      <c r="P49" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q49" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R49" s="3">
+        <v>0</v>
       </c>
       <c r="S49" s="3">
-        <v>1</v>
-      </c>
-      <c r="T49" s="3">
-        <v>1</v>
-      </c>
-      <c r="U49" s="3">
+        <v>0</v>
+      </c>
+      <c r="T49" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U49" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V49" s="3">
+        <v>1</v>
+      </c>
+      <c r="W49" s="3">
+        <v>1</v>
+      </c>
+      <c r="X49" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y49" s="3">
         <v>22</v>
       </c>
     </row>
-    <row r="50" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="50" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D50" s="16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E50" s="3">
         <v>1010011</v>
@@ -4019,8 +4610,8 @@
       <c r="I50" s="3">
         <v>0</v>
       </c>
-      <c r="J50" s="3">
-        <v>110</v>
+      <c r="J50" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K50" s="3">
         <v>0</v>
@@ -4034,31 +4625,43 @@
       <c r="N50" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O50" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P50" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q50" s="3">
-        <v>0</v>
-      </c>
-      <c r="R50" s="3" t="s">
-        <v>46</v>
+      <c r="O50" s="3">
+        <v>10</v>
+      </c>
+      <c r="P50" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q50" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R50" s="3">
+        <v>0</v>
       </c>
       <c r="S50" s="3">
-        <v>1</v>
-      </c>
-      <c r="T50" s="3">
-        <v>1</v>
-      </c>
-      <c r="U50" s="3">
+        <v>0</v>
+      </c>
+      <c r="T50" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U50" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V50" s="3">
+        <v>1</v>
+      </c>
+      <c r="W50" s="3">
+        <v>1</v>
+      </c>
+      <c r="X50" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y50" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="51" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D51" s="16" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E51" s="3">
         <v>1010011</v>
@@ -4075,8 +4678,8 @@
       <c r="I51" s="3">
         <v>0</v>
       </c>
-      <c r="J51" s="3">
-        <v>110</v>
+      <c r="J51" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K51" s="3">
         <v>0</v>
@@ -4090,31 +4693,43 @@
       <c r="N51" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O51" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P51" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q51" s="3">
-        <v>0</v>
-      </c>
-      <c r="R51" s="3" t="s">
-        <v>46</v>
+      <c r="O51" s="3">
+        <v>10</v>
+      </c>
+      <c r="P51" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q51" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R51" s="3">
+        <v>0</v>
       </c>
       <c r="S51" s="3">
-        <v>1</v>
-      </c>
-      <c r="T51" s="3">
-        <v>1</v>
-      </c>
-      <c r="U51" s="3">
+        <v>0</v>
+      </c>
+      <c r="T51" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U51" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V51" s="3">
+        <v>1</v>
+      </c>
+      <c r="W51" s="3">
+        <v>1</v>
+      </c>
+      <c r="X51" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y51" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="52" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="52" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D52" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E52" s="3">
         <v>1010011</v>
@@ -4131,8 +4746,8 @@
       <c r="I52" s="3">
         <v>0</v>
       </c>
-      <c r="J52" s="3">
-        <v>110</v>
+      <c r="J52" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K52" s="3">
         <v>0</v>
@@ -4146,31 +4761,43 @@
       <c r="N52" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O52" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P52" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q52" s="3">
-        <v>0</v>
-      </c>
-      <c r="R52" s="3" t="s">
-        <v>46</v>
+      <c r="O52" s="3">
+        <v>10</v>
+      </c>
+      <c r="P52" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q52" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R52" s="3">
+        <v>0</v>
       </c>
       <c r="S52" s="3">
-        <v>1</v>
-      </c>
-      <c r="T52" s="3">
-        <v>1</v>
-      </c>
-      <c r="U52" s="3">
+        <v>0</v>
+      </c>
+      <c r="T52" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U52" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V52" s="3">
+        <v>1</v>
+      </c>
+      <c r="W52" s="3">
+        <v>1</v>
+      </c>
+      <c r="X52" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y52" s="3">
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="4:21" x14ac:dyDescent="0.3">
+    <row r="53" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D53" s="16" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E53" s="3">
         <v>1010011</v>
@@ -4187,8 +4814,8 @@
       <c r="I53" s="3">
         <v>0</v>
       </c>
-      <c r="J53" s="3">
-        <v>110</v>
+      <c r="J53" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="K53" s="3">
         <v>0</v>
@@ -4202,45 +4829,60 @@
       <c r="N53" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O53" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P53" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q53" s="3">
-        <v>0</v>
-      </c>
-      <c r="R53" s="3" t="s">
-        <v>46</v>
+      <c r="O53" s="3">
+        <v>10</v>
+      </c>
+      <c r="P53" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q53" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R53" s="3">
+        <v>0</v>
       </c>
       <c r="S53" s="3">
-        <v>1</v>
-      </c>
-      <c r="T53" s="3">
-        <v>1</v>
-      </c>
-      <c r="U53" s="3">
+        <v>0</v>
+      </c>
+      <c r="T53" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U53" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V53" s="3">
+        <v>1</v>
+      </c>
+      <c r="W53" s="3">
+        <v>1</v>
+      </c>
+      <c r="X53" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y53" s="3">
         <v>2</v>
       </c>
+    </row>
+    <row r="54" spans="4:25" x14ac:dyDescent="0.3">
+      <c r="J54" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="D3:U3"/>
-    <mergeCell ref="W7:W11"/>
-    <mergeCell ref="W25:W32"/>
-    <mergeCell ref="AE9:AH9"/>
-    <mergeCell ref="AD23:AF23"/>
-    <mergeCell ref="AG23:AJ23"/>
-    <mergeCell ref="AD22:AF22"/>
-    <mergeCell ref="AG22:AJ22"/>
-    <mergeCell ref="AD26:AE26"/>
-    <mergeCell ref="AD27:AE27"/>
-    <mergeCell ref="AD28:AE28"/>
-    <mergeCell ref="AF25:AI25"/>
-    <mergeCell ref="AF26:AI26"/>
-    <mergeCell ref="AF27:AI27"/>
-    <mergeCell ref="AF28:AI28"/>
+    <mergeCell ref="D3:Y3"/>
+    <mergeCell ref="AA7:AA11"/>
+    <mergeCell ref="AA25:AA32"/>
+    <mergeCell ref="AI9:AL9"/>
+    <mergeCell ref="AH23:AJ23"/>
+    <mergeCell ref="AK23:AN23"/>
+    <mergeCell ref="AH22:AJ22"/>
+    <mergeCell ref="AK22:AN22"/>
+    <mergeCell ref="AH26:AI26"/>
+    <mergeCell ref="AH27:AI27"/>
+    <mergeCell ref="AH28:AI28"/>
+    <mergeCell ref="AJ25:AM25"/>
+    <mergeCell ref="AJ26:AM26"/>
+    <mergeCell ref="AJ27:AM27"/>
+    <mergeCell ref="AJ28:AM28"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4449,20 +5091,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="aa762089-36ad-4bf7-9314-c7223c4b604d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="aa762089-36ad-4bf7-9314-c7223c4b604d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4484,14 +5126,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A7B8669E-67F1-4457-BB68-A16754986870}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E0D4C47-9B8A-40A7-B507-77A4C6E21046}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -4505,4 +5139,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A7B8669E-67F1-4457-BB68-A16754986870}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update control for RV32IMF
</commit_message>
<xml_diff>
--- a/Control.xlsx
+++ b/Control.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Hung\Khoa_Luan\ISS-RV32ICMFA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE8BC07F-AB9F-45B5-9510-7506420B6DDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A3298FA-14F9-4BCE-BAF9-344F73BED60E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CF86E8A2-CD57-4282-A2FF-4C2B018B82AC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="137">
   <si>
     <t>instructions</t>
   </si>
@@ -411,49 +411,55 @@
     <t>0100111</t>
   </si>
   <si>
+    <t>xxxxx</t>
+  </si>
+  <si>
+    <t>mulhsu</t>
+  </si>
+  <si>
+    <t>mulhu</t>
+  </si>
+  <si>
+    <t>divu</t>
+  </si>
+  <si>
+    <t>Mul_Div_unsigned</t>
+  </si>
+  <si>
+    <t>valid_MDU</t>
+  </si>
+  <si>
+    <t>z0</t>
+  </si>
+  <si>
+    <t>z1</t>
+  </si>
+  <si>
+    <t>addr_addend_sel</t>
+  </si>
+  <si>
+    <t>ResExSel</t>
+  </si>
+  <si>
+    <t>ResPCSel</t>
+  </si>
+  <si>
+    <t>Valid_FPU</t>
+  </si>
+  <si>
+    <t>RegSrc1</t>
+  </si>
+  <si>
+    <t>RegSrc2</t>
+  </si>
+  <si>
+    <t>MulDivControl</t>
+  </si>
+  <si>
+    <t>FPUControl</t>
+  </si>
+  <si>
     <t>FPUOp</t>
-  </si>
-  <si>
-    <t>xxxxx</t>
-  </si>
-  <si>
-    <t>mulhsu</t>
-  </si>
-  <si>
-    <t>mulhu</t>
-  </si>
-  <si>
-    <t>divu</t>
-  </si>
-  <si>
-    <t>Mul_Div_unsigned</t>
-  </si>
-  <si>
-    <t>valid_MDU</t>
-  </si>
-  <si>
-    <t>z0</t>
-  </si>
-  <si>
-    <t>z1</t>
-  </si>
-  <si>
-    <t>addr_addend_sel</t>
-  </si>
-  <si>
-    <t>ResExSel</t>
-  </si>
-  <si>
-    <t>ResPCSel</t>
-  </si>
-  <si>
-    <t>Valid_FPU</t>
-  </si>
-  <si>
-    <t>RegSrc1</t>
-  </si>
-  <si>
-    <t>RegSrc2</t>
   </si>
 </sst>
 </file>
@@ -533,7 +539,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -639,11 +645,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -690,6 +705,18 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -720,16 +747,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1073,6 +1097,7 @@
     <col min="14" max="16" width="16.33203125" customWidth="1"/>
     <col min="17" max="17" width="18.109375" customWidth="1"/>
     <col min="18" max="18" width="10.33203125" customWidth="1"/>
+    <col min="19" max="19" width="15" customWidth="1"/>
     <col min="21" max="21" width="8.88671875" customWidth="1"/>
     <col min="22" max="22" width="9" customWidth="1"/>
     <col min="23" max="23" width="10.6640625" customWidth="1"/>
@@ -1086,31 +1111,31 @@
   </cols>
   <sheetData>
     <row r="3" spans="4:41" x14ac:dyDescent="0.3">
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17"/>
-      <c r="M3" s="17"/>
-      <c r="N3" s="17"/>
-      <c r="O3" s="17"/>
-      <c r="P3" s="17"/>
-      <c r="Q3" s="17"/>
-      <c r="R3" s="17"/>
-      <c r="S3" s="17"/>
-      <c r="T3" s="17"/>
-      <c r="U3" s="17"/>
-      <c r="V3" s="17"/>
-      <c r="W3" s="17"/>
-      <c r="X3" s="17"/>
-      <c r="Y3" s="17"/>
-      <c r="Z3" s="18"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="21"/>
+      <c r="P3" s="21"/>
+      <c r="Q3" s="21"/>
+      <c r="R3" s="21"/>
+      <c r="S3" s="21"/>
+      <c r="T3" s="21"/>
+      <c r="U3" s="21"/>
+      <c r="V3" s="21"/>
+      <c r="W3" s="21"/>
+      <c r="X3" s="21"/>
+      <c r="Y3" s="21"/>
+      <c r="Z3" s="22"/>
       <c r="AB3" t="s">
         <v>17</v>
       </c>
@@ -1147,22 +1172,22 @@
         <v>42</v>
       </c>
       <c r="N4" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="O4" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="O4" s="3" t="s">
+      <c r="P4" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="P4" s="3" t="s">
-        <v>131</v>
-      </c>
       <c r="Q4" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="R4" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="R4" s="3" t="s">
-        <v>126</v>
-      </c>
       <c r="S4" s="3" t="s">
-        <v>53</v>
+        <v>134</v>
       </c>
       <c r="T4" s="3" t="s">
         <v>56</v>
@@ -1174,16 +1199,16 @@
         <v>91</v>
       </c>
       <c r="W4" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="X4" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="X4" s="3" t="s">
+      <c r="Y4" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="Y4" s="3" t="s">
-        <v>134</v>
-      </c>
       <c r="Z4" s="3" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="AB4" s="1" t="s">
         <v>11</v>
@@ -1262,14 +1287,14 @@
       <c r="W5" s="3">
         <v>0</v>
       </c>
-      <c r="X5" s="3" t="s">
-        <v>16</v>
+      <c r="X5" s="3">
+        <v>0</v>
       </c>
       <c r="Y5" s="3" t="s">
         <v>16</v>
       </c>
       <c r="Z5" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AB5" s="2" t="s">
         <v>13</v>
@@ -1355,7 +1380,7 @@
         <v>0</v>
       </c>
       <c r="Z6" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AB6" s="2" t="s">
         <v>14</v>
@@ -1441,9 +1466,9 @@
         <v>0</v>
       </c>
       <c r="Z7" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="AB7" s="19">
+        <v>120</v>
+      </c>
+      <c r="AB7" s="23">
         <v>10</v>
       </c>
       <c r="AC7" s="2" t="s">
@@ -1527,9 +1552,9 @@
         <v>0</v>
       </c>
       <c r="Z8" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="AB8" s="20"/>
+        <v>120</v>
+      </c>
+      <c r="AB8" s="24"/>
       <c r="AC8" s="2" t="s">
         <v>25</v>
       </c>
@@ -1556,8 +1581,8 @@
       <c r="G9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H9" s="3" t="s">
-        <v>16</v>
+      <c r="H9" s="3">
+        <v>1</v>
       </c>
       <c r="I9" s="3">
         <v>0</v>
@@ -1611,9 +1636,9 @@
         <v>0</v>
       </c>
       <c r="Z9" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="AB9" s="20"/>
+        <v>120</v>
+      </c>
+      <c r="AB9" s="24"/>
       <c r="AC9" s="2" t="s">
         <v>26</v>
       </c>
@@ -1632,12 +1657,12 @@
       <c r="AI9" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="AJ9" s="23" t="s">
+      <c r="AJ9" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="AK9" s="23"/>
-      <c r="AL9" s="23"/>
-      <c r="AM9" s="23"/>
+      <c r="AK9" s="27"/>
+      <c r="AL9" s="27"/>
+      <c r="AM9" s="27"/>
       <c r="AN9" s="1" t="s">
         <v>75</v>
       </c>
@@ -1713,9 +1738,9 @@
         <v>0</v>
       </c>
       <c r="Z10" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="AB10" s="20"/>
+        <v>120</v>
+      </c>
+      <c r="AB10" s="24"/>
       <c r="AC10" s="1">
         <v>110</v>
       </c>
@@ -1758,7 +1783,7 @@
         <v>1</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>16</v>
@@ -1815,9 +1840,9 @@
         <v>0</v>
       </c>
       <c r="Z11" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="AB11" s="21"/>
+        <v>120</v>
+      </c>
+      <c r="AB11" s="25"/>
       <c r="AC11" s="1">
         <v>111</v>
       </c>
@@ -1899,7 +1924,7 @@
         <v>0</v>
       </c>
       <c r="Z12" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="13" spans="4:41" x14ac:dyDescent="0.3">
@@ -1970,7 +1995,7 @@
         <v>0</v>
       </c>
       <c r="Z13" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="14" spans="4:41" x14ac:dyDescent="0.3">
@@ -2041,7 +2066,7 @@
         <v>0</v>
       </c>
       <c r="Z14" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" spans="4:41" x14ac:dyDescent="0.3">
@@ -2112,12 +2137,12 @@
         <v>0</v>
       </c>
       <c r="Z15" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" spans="4:41" x14ac:dyDescent="0.3">
       <c r="D16" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>39</v>
@@ -2183,12 +2208,12 @@
         <v>0</v>
       </c>
       <c r="Z16" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17" spans="4:41" x14ac:dyDescent="0.3">
       <c r="D17" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>39</v>
@@ -2254,7 +2279,7 @@
         <v>0</v>
       </c>
       <c r="Z17" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18" spans="4:41" x14ac:dyDescent="0.3">
@@ -2298,7 +2323,7 @@
         <v>16</v>
       </c>
       <c r="Q18" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="R18" s="5">
         <v>1</v>
@@ -2325,12 +2350,12 @@
         <v>0</v>
       </c>
       <c r="Z18" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" spans="4:41" x14ac:dyDescent="0.3">
       <c r="D19" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>39</v>
@@ -2369,7 +2394,7 @@
         <v>16</v>
       </c>
       <c r="Q19" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="R19" s="5">
         <v>1</v>
@@ -2396,7 +2421,7 @@
         <v>0</v>
       </c>
       <c r="Z19" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="20" spans="4:41" x14ac:dyDescent="0.3">
@@ -2440,7 +2465,7 @@
         <v>16</v>
       </c>
       <c r="Q20" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="R20" s="5">
         <v>1</v>
@@ -2467,7 +2492,7 @@
         <v>0</v>
       </c>
       <c r="Z20" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="21" spans="4:41" x14ac:dyDescent="0.3">
@@ -2511,7 +2536,7 @@
         <v>16</v>
       </c>
       <c r="Q21" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="R21" s="5">
         <v>1</v>
@@ -2538,7 +2563,7 @@
         <v>0</v>
       </c>
       <c r="Z21" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="22" spans="4:41" x14ac:dyDescent="0.3">
@@ -2609,7 +2634,7 @@
         <v>0</v>
       </c>
       <c r="Z22" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AB22" t="s">
         <v>54</v>
@@ -2617,17 +2642,17 @@
       <c r="AH22" t="s">
         <v>77</v>
       </c>
-      <c r="AI22" s="24" t="s">
+      <c r="AI22" s="28" t="s">
         <v>81</v>
       </c>
-      <c r="AJ22" s="24"/>
-      <c r="AK22" s="24"/>
-      <c r="AL22" s="24" t="s">
+      <c r="AJ22" s="28"/>
+      <c r="AK22" s="28"/>
+      <c r="AL22" s="28" t="s">
         <v>82</v>
       </c>
-      <c r="AM22" s="24"/>
-      <c r="AN22" s="24"/>
-      <c r="AO22" s="24"/>
+      <c r="AM22" s="28"/>
+      <c r="AN22" s="28"/>
+      <c r="AO22" s="28"/>
     </row>
     <row r="23" spans="4:41" x14ac:dyDescent="0.3">
       <c r="D23" s="11" t="s">
@@ -2697,7 +2722,7 @@
         <v>0</v>
       </c>
       <c r="Z23" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AB23" s="1" t="s">
         <v>53</v>
@@ -2717,17 +2742,17 @@
       <c r="AH23" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="AI23" s="23" t="s">
+      <c r="AI23" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="AJ23" s="23"/>
-      <c r="AK23" s="23"/>
-      <c r="AL23" s="23" t="s">
+      <c r="AJ23" s="27"/>
+      <c r="AK23" s="27"/>
+      <c r="AL23" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="AM23" s="23"/>
-      <c r="AN23" s="23"/>
-      <c r="AO23" s="23"/>
+      <c r="AM23" s="27"/>
+      <c r="AN23" s="27"/>
+      <c r="AO23" s="27"/>
     </row>
     <row r="24" spans="4:41" x14ac:dyDescent="0.3">
       <c r="D24" s="11" t="s">
@@ -2797,7 +2822,7 @@
         <v>0</v>
       </c>
       <c r="Z24" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AB24" s="2">
         <v>0</v>
@@ -2883,9 +2908,9 @@
         <v>0</v>
       </c>
       <c r="Z25" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="AB25" s="22">
+        <v>120</v>
+      </c>
+      <c r="AB25" s="26">
         <v>1</v>
       </c>
       <c r="AC25" s="1">
@@ -2907,12 +2932,12 @@
         <v>84</v>
       </c>
       <c r="AJ25" s="3"/>
-      <c r="AK25" s="25" t="s">
+      <c r="AK25" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="AL25" s="25"/>
-      <c r="AM25" s="25"/>
-      <c r="AN25" s="25"/>
+      <c r="AL25" s="29"/>
+      <c r="AM25" s="29"/>
+      <c r="AN25" s="29"/>
     </row>
     <row r="26" spans="4:41" x14ac:dyDescent="0.3">
       <c r="D26" s="15" t="s">
@@ -2982,9 +3007,9 @@
         <v>0</v>
       </c>
       <c r="Z26" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="AB26" s="22"/>
+        <v>120</v>
+      </c>
+      <c r="AB26" s="26"/>
       <c r="AC26" s="2">
         <v>1</v>
       </c>
@@ -3000,16 +3025,16 @@
       <c r="AH26" s="3">
         <v>0</v>
       </c>
-      <c r="AI26" s="25">
+      <c r="AI26" s="29">
         <v>-127</v>
       </c>
-      <c r="AJ26" s="25"/>
-      <c r="AK26" s="25" t="s">
+      <c r="AJ26" s="29"/>
+      <c r="AK26" s="29" t="s">
         <v>88</v>
       </c>
-      <c r="AL26" s="25"/>
-      <c r="AM26" s="25"/>
-      <c r="AN26" s="25"/>
+      <c r="AL26" s="29"/>
+      <c r="AM26" s="29"/>
+      <c r="AN26" s="29"/>
     </row>
     <row r="27" spans="4:41" x14ac:dyDescent="0.3">
       <c r="D27" s="15" t="s">
@@ -3079,9 +3104,9 @@
         <v>0</v>
       </c>
       <c r="Z27" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="AB27" s="22"/>
+        <v>120</v>
+      </c>
+      <c r="AB27" s="26"/>
       <c r="AC27" s="2">
         <v>2</v>
       </c>
@@ -3097,88 +3122,88 @@
       <c r="AH27" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="AI27" s="22" t="s">
+      <c r="AI27" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="AJ27" s="22"/>
-      <c r="AK27" s="25" t="s">
+      <c r="AJ27" s="26"/>
+      <c r="AK27" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="AL27" s="25"/>
-      <c r="AM27" s="25"/>
-      <c r="AN27" s="25"/>
+      <c r="AL27" s="29"/>
+      <c r="AM27" s="29"/>
+      <c r="AN27" s="29"/>
     </row>
     <row r="28" spans="4:41" x14ac:dyDescent="0.3">
-      <c r="D28" s="26" t="s">
+      <c r="D28" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="E28" s="27" t="s">
+      <c r="E28" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="F28" s="26">
-        <v>0</v>
-      </c>
-      <c r="G28" s="27" t="s">
+      <c r="F28" s="16">
+        <v>0</v>
+      </c>
+      <c r="G28" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="H28" s="26">
-        <v>1</v>
-      </c>
-      <c r="I28" s="26">
-        <v>0</v>
-      </c>
-      <c r="J28" s="27" t="s">
+      <c r="H28" s="16">
+        <v>1</v>
+      </c>
+      <c r="I28" s="16">
+        <v>0</v>
+      </c>
+      <c r="J28" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="K28" s="26">
-        <v>0</v>
-      </c>
-      <c r="L28" s="27" t="s">
+      <c r="K28" s="16">
+        <v>0</v>
+      </c>
+      <c r="L28" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="M28" s="26">
-        <v>0</v>
-      </c>
-      <c r="N28" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O28" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="P28" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q28" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R28" s="26">
-        <v>0</v>
-      </c>
-      <c r="S28" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T28" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U28" s="27" t="s">
+      <c r="M28" s="16">
+        <v>0</v>
+      </c>
+      <c r="N28" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O28" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="P28" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q28" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R28" s="16">
+        <v>0</v>
+      </c>
+      <c r="S28" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T28" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U28" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="V28" s="26">
-        <v>1</v>
-      </c>
-      <c r="W28" s="26">
-        <v>0</v>
-      </c>
-      <c r="X28" s="26">
-        <v>0</v>
-      </c>
-      <c r="Y28" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Z28" s="26" t="s">
-        <v>121</v>
-      </c>
-      <c r="AB28" s="22"/>
+      <c r="V28" s="16">
+        <v>1</v>
+      </c>
+      <c r="W28" s="16">
+        <v>0</v>
+      </c>
+      <c r="X28" s="16">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z28" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="AB28" s="26"/>
       <c r="AC28" s="2">
         <v>3</v>
       </c>
@@ -3194,93 +3219,93 @@
       <c r="AH28" s="3">
         <v>255</v>
       </c>
-      <c r="AI28" s="25">
+      <c r="AI28" s="29">
         <v>128</v>
       </c>
-      <c r="AJ28" s="25"/>
-      <c r="AK28" s="25" t="s">
+      <c r="AJ28" s="29"/>
+      <c r="AK28" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="AL28" s="25"/>
-      <c r="AM28" s="25"/>
-      <c r="AN28" s="25"/>
+      <c r="AL28" s="29"/>
+      <c r="AM28" s="29"/>
+      <c r="AN28" s="29"/>
     </row>
     <row r="29" spans="4:41" x14ac:dyDescent="0.3">
-      <c r="D29" s="26" t="s">
+      <c r="D29" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="E29" s="27" t="s">
+      <c r="E29" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="F29" s="26">
-        <v>0</v>
-      </c>
-      <c r="G29" s="27" t="s">
+      <c r="F29" s="16">
+        <v>0</v>
+      </c>
+      <c r="G29" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="H29" s="26">
-        <v>1</v>
-      </c>
-      <c r="I29" s="26">
-        <v>1</v>
-      </c>
-      <c r="J29" s="27" t="s">
+      <c r="H29" s="16">
+        <v>1</v>
+      </c>
+      <c r="I29" s="16">
+        <v>1</v>
+      </c>
+      <c r="J29" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K29" s="26">
-        <v>0</v>
-      </c>
-      <c r="L29" s="27" t="s">
+      <c r="K29" s="16">
+        <v>0</v>
+      </c>
+      <c r="L29" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="M29" s="26">
-        <v>0</v>
-      </c>
-      <c r="N29" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O29" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="P29" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q29" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R29" s="26">
-        <v>0</v>
-      </c>
-      <c r="S29" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T29" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U29" s="27" t="s">
+      <c r="M29" s="16">
+        <v>0</v>
+      </c>
+      <c r="N29" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O29" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="P29" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q29" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R29" s="16">
+        <v>0</v>
+      </c>
+      <c r="S29" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T29" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U29" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="V29" s="26">
-        <v>0</v>
-      </c>
-      <c r="W29" s="26">
-        <v>0</v>
-      </c>
-      <c r="X29" s="26">
-        <v>0</v>
-      </c>
-      <c r="Y29" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z29" s="26" t="s">
-        <v>121</v>
-      </c>
-      <c r="AB29" s="22"/>
+      <c r="V29" s="16">
+        <v>0</v>
+      </c>
+      <c r="W29" s="16">
+        <v>0</v>
+      </c>
+      <c r="X29" s="16">
+        <v>0</v>
+      </c>
+      <c r="Y29" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z29" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="AB29" s="26"/>
       <c r="AC29" s="1">
         <v>4</v>
       </c>
       <c r="AD29" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AE29" s="1" t="s">
         <v>16</v>
@@ -3290,81 +3315,81 @@
       </c>
     </row>
     <row r="30" spans="4:41" x14ac:dyDescent="0.3">
-      <c r="D30" s="28" t="s">
+      <c r="D30" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="E30" s="28">
+      <c r="E30" s="18">
         <v>1000011</v>
       </c>
-      <c r="F30" s="28">
-        <v>0</v>
-      </c>
-      <c r="G30" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="H30" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="I30" s="28">
-        <v>0</v>
-      </c>
-      <c r="J30" s="29" t="s">
+      <c r="F30" s="18">
+        <v>0</v>
+      </c>
+      <c r="G30" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="H30" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="I30" s="18">
+        <v>0</v>
+      </c>
+      <c r="J30" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="K30" s="28">
-        <v>0</v>
-      </c>
-      <c r="L30" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="M30" s="28">
-        <v>0</v>
-      </c>
-      <c r="N30" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="O30" s="28">
+      <c r="K30" s="18">
+        <v>0</v>
+      </c>
+      <c r="L30" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="M30" s="18">
+        <v>0</v>
+      </c>
+      <c r="N30" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="O30" s="18">
         <v>10</v>
       </c>
-      <c r="P30" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q30" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="R30" s="28">
-        <v>0</v>
-      </c>
-      <c r="S30" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="T30" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="U30" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="V30" s="28">
-        <v>1</v>
-      </c>
-      <c r="W30" s="28">
-        <v>1</v>
-      </c>
-      <c r="X30" s="28">
-        <v>1</v>
-      </c>
-      <c r="Y30" s="28">
-        <v>1</v>
-      </c>
-      <c r="Z30" s="28">
+      <c r="P30" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q30" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="R30" s="18">
+        <v>0</v>
+      </c>
+      <c r="S30" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="T30" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="U30" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="V30" s="18">
+        <v>1</v>
+      </c>
+      <c r="W30" s="18">
+        <v>1</v>
+      </c>
+      <c r="X30" s="18">
+        <v>1</v>
+      </c>
+      <c r="Y30" s="18">
+        <v>1</v>
+      </c>
+      <c r="Z30" s="18">
         <v>11</v>
       </c>
-      <c r="AB30" s="22"/>
+      <c r="AB30" s="26"/>
       <c r="AC30" s="1">
         <v>5</v>
       </c>
       <c r="AD30" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AE30" s="1" t="s">
         <v>16</v>
@@ -3374,81 +3399,81 @@
       </c>
     </row>
     <row r="31" spans="4:41" x14ac:dyDescent="0.3">
-      <c r="D31" s="28" t="s">
+      <c r="D31" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="E31" s="28">
+      <c r="E31" s="18">
         <v>1000111</v>
       </c>
-      <c r="F31" s="28">
-        <v>0</v>
-      </c>
-      <c r="G31" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="H31" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="I31" s="28">
-        <v>0</v>
-      </c>
-      <c r="J31" s="29" t="s">
+      <c r="F31" s="18">
+        <v>0</v>
+      </c>
+      <c r="G31" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="H31" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="I31" s="18">
+        <v>0</v>
+      </c>
+      <c r="J31" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="K31" s="28">
-        <v>0</v>
-      </c>
-      <c r="L31" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="M31" s="28">
-        <v>0</v>
-      </c>
-      <c r="N31" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="O31" s="28">
+      <c r="K31" s="18">
+        <v>0</v>
+      </c>
+      <c r="L31" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="M31" s="18">
+        <v>0</v>
+      </c>
+      <c r="N31" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="O31" s="18">
         <v>10</v>
       </c>
-      <c r="P31" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q31" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="R31" s="28">
-        <v>0</v>
-      </c>
-      <c r="S31" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="T31" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="U31" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="V31" s="28">
-        <v>1</v>
-      </c>
-      <c r="W31" s="28">
-        <v>1</v>
-      </c>
-      <c r="X31" s="28">
-        <v>1</v>
-      </c>
-      <c r="Y31" s="28">
-        <v>1</v>
-      </c>
-      <c r="Z31" s="28">
+      <c r="P31" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q31" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="R31" s="18">
+        <v>0</v>
+      </c>
+      <c r="S31" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="T31" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="U31" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="V31" s="18">
+        <v>1</v>
+      </c>
+      <c r="W31" s="18">
+        <v>1</v>
+      </c>
+      <c r="X31" s="18">
+        <v>1</v>
+      </c>
+      <c r="Y31" s="18">
+        <v>1</v>
+      </c>
+      <c r="Z31" s="18">
         <v>12</v>
       </c>
-      <c r="AB31" s="22"/>
+      <c r="AB31" s="26"/>
       <c r="AC31" s="1">
         <v>6</v>
       </c>
       <c r="AD31" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AE31" s="1" t="s">
         <v>16</v>
@@ -3458,81 +3483,81 @@
       </c>
     </row>
     <row r="32" spans="4:41" x14ac:dyDescent="0.3">
-      <c r="D32" s="28" t="s">
+      <c r="D32" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="E32" s="28">
+      <c r="E32" s="18">
         <v>1001111</v>
       </c>
-      <c r="F32" s="28">
-        <v>0</v>
-      </c>
-      <c r="G32" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="H32" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="I32" s="28">
-        <v>0</v>
-      </c>
-      <c r="J32" s="29" t="s">
+      <c r="F32" s="18">
+        <v>0</v>
+      </c>
+      <c r="G32" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="H32" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="I32" s="18">
+        <v>0</v>
+      </c>
+      <c r="J32" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="K32" s="28">
-        <v>0</v>
-      </c>
-      <c r="L32" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="M32" s="28">
-        <v>0</v>
-      </c>
-      <c r="N32" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="O32" s="28">
+      <c r="K32" s="18">
+        <v>0</v>
+      </c>
+      <c r="L32" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="M32" s="18">
+        <v>0</v>
+      </c>
+      <c r="N32" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="O32" s="18">
         <v>10</v>
       </c>
-      <c r="P32" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q32" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="R32" s="28">
-        <v>0</v>
-      </c>
-      <c r="S32" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="T32" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="U32" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="V32" s="28">
-        <v>1</v>
-      </c>
-      <c r="W32" s="28">
-        <v>1</v>
-      </c>
-      <c r="X32" s="28">
-        <v>1</v>
-      </c>
-      <c r="Y32" s="28">
-        <v>1</v>
-      </c>
-      <c r="Z32" s="28">
+      <c r="P32" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q32" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="R32" s="18">
+        <v>0</v>
+      </c>
+      <c r="S32" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="T32" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="U32" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="V32" s="18">
+        <v>1</v>
+      </c>
+      <c r="W32" s="18">
+        <v>1</v>
+      </c>
+      <c r="X32" s="18">
+        <v>1</v>
+      </c>
+      <c r="Y32" s="18">
+        <v>1</v>
+      </c>
+      <c r="Z32" s="18">
         <v>13</v>
       </c>
-      <c r="AB32" s="22"/>
+      <c r="AB32" s="26"/>
       <c r="AC32" s="1">
         <v>7</v>
       </c>
       <c r="AD32" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AE32" s="1" t="s">
         <v>16</v>
@@ -3541,1494 +3566,1515 @@
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D33" s="28" t="s">
+    <row r="33" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D33" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="E33" s="28">
+      <c r="E33" s="18">
         <v>1001011</v>
       </c>
-      <c r="F33" s="28">
-        <v>0</v>
-      </c>
-      <c r="G33" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="H33" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="I33" s="28">
-        <v>0</v>
-      </c>
-      <c r="J33" s="29" t="s">
+      <c r="F33" s="18">
+        <v>0</v>
+      </c>
+      <c r="G33" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="H33" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="I33" s="18">
+        <v>0</v>
+      </c>
+      <c r="J33" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="K33" s="28">
-        <v>0</v>
-      </c>
-      <c r="L33" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="M33" s="28">
-        <v>0</v>
-      </c>
-      <c r="N33" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="O33" s="28">
+      <c r="K33" s="18">
+        <v>0</v>
+      </c>
+      <c r="L33" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="M33" s="18">
+        <v>0</v>
+      </c>
+      <c r="N33" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="O33" s="18">
         <v>10</v>
       </c>
-      <c r="P33" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q33" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="R33" s="28">
-        <v>0</v>
-      </c>
-      <c r="S33" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="T33" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="U33" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="V33" s="28">
-        <v>1</v>
-      </c>
-      <c r="W33" s="28">
-        <v>1</v>
-      </c>
-      <c r="X33" s="28">
-        <v>1</v>
-      </c>
-      <c r="Y33" s="28">
-        <v>1</v>
-      </c>
-      <c r="Z33" s="28">
+      <c r="P33" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q33" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="R33" s="18">
+        <v>0</v>
+      </c>
+      <c r="S33" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="T33" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="U33" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="V33" s="18">
+        <v>1</v>
+      </c>
+      <c r="W33" s="18">
+        <v>1</v>
+      </c>
+      <c r="X33" s="18">
+        <v>1</v>
+      </c>
+      <c r="Y33" s="18">
+        <v>1</v>
+      </c>
+      <c r="Z33" s="18">
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D34" s="26" t="s">
+    <row r="34" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D34" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="E34" s="26">
+      <c r="E34" s="16">
         <v>1010011</v>
       </c>
-      <c r="F34" s="26">
-        <v>0</v>
-      </c>
-      <c r="G34" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H34" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I34" s="26">
-        <v>0</v>
-      </c>
-      <c r="J34" s="27" t="s">
+      <c r="F34" s="16">
+        <v>0</v>
+      </c>
+      <c r="G34" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H34" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I34" s="16">
+        <v>0</v>
+      </c>
+      <c r="J34" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K34" s="26">
-        <v>0</v>
-      </c>
-      <c r="L34" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M34" s="26">
-        <v>0</v>
-      </c>
-      <c r="N34" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O34" s="26">
+      <c r="K34" s="16">
+        <v>0</v>
+      </c>
+      <c r="L34" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M34" s="16">
+        <v>0</v>
+      </c>
+      <c r="N34" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O34" s="16">
         <v>10</v>
       </c>
-      <c r="P34" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q34" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R34" s="26">
-        <v>0</v>
-      </c>
-      <c r="S34" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T34" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U34" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V34" s="26">
-        <v>1</v>
-      </c>
-      <c r="W34" s="26">
-        <v>1</v>
-      </c>
-      <c r="X34" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y34" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z34" s="26">
+      <c r="P34" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q34" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R34" s="16">
+        <v>0</v>
+      </c>
+      <c r="S34" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T34" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U34" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V34" s="16">
+        <v>1</v>
+      </c>
+      <c r="W34" s="16">
+        <v>1</v>
+      </c>
+      <c r="X34" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y34" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z34" s="16">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D35" s="26" t="s">
+    <row r="35" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D35" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="E35" s="26">
+      <c r="E35" s="16">
         <v>1010011</v>
       </c>
-      <c r="F35" s="26">
-        <v>0</v>
-      </c>
-      <c r="G35" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H35" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I35" s="26">
-        <v>0</v>
-      </c>
-      <c r="J35" s="27" t="s">
+      <c r="F35" s="16">
+        <v>0</v>
+      </c>
+      <c r="G35" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H35" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I35" s="16">
+        <v>0</v>
+      </c>
+      <c r="J35" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K35" s="26">
-        <v>0</v>
-      </c>
-      <c r="L35" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M35" s="26">
-        <v>0</v>
-      </c>
-      <c r="N35" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O35" s="26">
+      <c r="K35" s="16">
+        <v>0</v>
+      </c>
+      <c r="L35" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M35" s="16">
+        <v>0</v>
+      </c>
+      <c r="N35" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O35" s="16">
         <v>10</v>
       </c>
-      <c r="P35" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q35" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R35" s="26">
-        <v>0</v>
-      </c>
-      <c r="S35" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T35" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U35" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V35" s="26">
-        <v>1</v>
-      </c>
-      <c r="W35" s="26">
-        <v>1</v>
-      </c>
-      <c r="X35" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y35" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z35" s="26">
+      <c r="P35" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q35" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R35" s="16">
+        <v>0</v>
+      </c>
+      <c r="S35" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T35" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U35" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V35" s="16">
+        <v>1</v>
+      </c>
+      <c r="W35" s="16">
+        <v>1</v>
+      </c>
+      <c r="X35" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y35" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z35" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D36" s="26" t="s">
+    <row r="36" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D36" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="E36" s="26">
+      <c r="E36" s="16">
         <v>1010011</v>
       </c>
-      <c r="F36" s="26">
-        <v>0</v>
-      </c>
-      <c r="G36" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H36" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I36" s="26">
-        <v>0</v>
-      </c>
-      <c r="J36" s="27" t="s">
+      <c r="F36" s="16">
+        <v>0</v>
+      </c>
+      <c r="G36" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H36" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I36" s="16">
+        <v>0</v>
+      </c>
+      <c r="J36" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K36" s="26">
-        <v>0</v>
-      </c>
-      <c r="L36" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M36" s="26">
-        <v>0</v>
-      </c>
-      <c r="N36" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O36" s="26">
+      <c r="K36" s="16">
+        <v>0</v>
+      </c>
+      <c r="L36" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M36" s="16">
+        <v>0</v>
+      </c>
+      <c r="N36" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O36" s="16">
         <v>10</v>
       </c>
-      <c r="P36" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q36" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R36" s="26">
-        <v>0</v>
-      </c>
-      <c r="S36" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T36" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U36" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V36" s="26">
-        <v>1</v>
-      </c>
-      <c r="W36" s="26">
-        <v>1</v>
-      </c>
-      <c r="X36" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y36" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z36" s="26">
+      <c r="P36" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q36" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R36" s="16">
+        <v>0</v>
+      </c>
+      <c r="S36" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T36" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U36" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V36" s="16">
+        <v>1</v>
+      </c>
+      <c r="W36" s="16">
+        <v>1</v>
+      </c>
+      <c r="X36" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y36" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z36" s="16">
         <v>17</v>
       </c>
     </row>
-    <row r="37" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D37" s="26" t="s">
+    <row r="37" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D37" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="E37" s="26">
+      <c r="E37" s="16">
         <v>1010011</v>
       </c>
-      <c r="F37" s="26">
-        <v>0</v>
-      </c>
-      <c r="G37" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H37" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I37" s="26">
-        <v>0</v>
-      </c>
-      <c r="J37" s="27" t="s">
+      <c r="F37" s="16">
+        <v>0</v>
+      </c>
+      <c r="G37" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H37" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I37" s="16">
+        <v>0</v>
+      </c>
+      <c r="J37" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K37" s="26">
-        <v>0</v>
-      </c>
-      <c r="L37" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M37" s="26">
-        <v>0</v>
-      </c>
-      <c r="N37" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O37" s="26">
+      <c r="K37" s="16">
+        <v>0</v>
+      </c>
+      <c r="L37" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M37" s="16">
+        <v>0</v>
+      </c>
+      <c r="N37" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O37" s="16">
         <v>10</v>
       </c>
-      <c r="P37" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q37" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R37" s="26">
-        <v>0</v>
-      </c>
-      <c r="S37" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T37" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U37" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V37" s="26">
-        <v>1</v>
-      </c>
-      <c r="W37" s="26">
-        <v>1</v>
-      </c>
-      <c r="X37" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y37" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z37" s="26">
+      <c r="P37" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q37" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R37" s="16">
+        <v>0</v>
+      </c>
+      <c r="S37" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T37" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U37" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V37" s="16">
+        <v>1</v>
+      </c>
+      <c r="W37" s="16">
+        <v>1</v>
+      </c>
+      <c r="X37" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y37" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z37" s="16">
         <v>7</v>
       </c>
+      <c r="AB37" t="s">
+        <v>136</v>
+      </c>
     </row>
-    <row r="38" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D38" s="26" t="s">
+    <row r="38" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D38" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="E38" s="26">
+      <c r="E38" s="16">
         <v>1010011</v>
       </c>
-      <c r="F38" s="26">
-        <v>0</v>
-      </c>
-      <c r="G38" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H38" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I38" s="26">
-        <v>0</v>
-      </c>
-      <c r="J38" s="27" t="s">
+      <c r="F38" s="16">
+        <v>0</v>
+      </c>
+      <c r="G38" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H38" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I38" s="16">
+        <v>0</v>
+      </c>
+      <c r="J38" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K38" s="26">
-        <v>0</v>
-      </c>
-      <c r="L38" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M38" s="26">
-        <v>0</v>
-      </c>
-      <c r="N38" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O38" s="26">
+      <c r="K38" s="16">
+        <v>0</v>
+      </c>
+      <c r="L38" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M38" s="16">
+        <v>0</v>
+      </c>
+      <c r="N38" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O38" s="16">
         <v>10</v>
       </c>
-      <c r="P38" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q38" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R38" s="26">
-        <v>0</v>
-      </c>
-      <c r="S38" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T38" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U38" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V38" s="26">
-        <v>1</v>
-      </c>
-      <c r="W38" s="26">
-        <v>1</v>
-      </c>
-      <c r="X38" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y38" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z38" s="26">
+      <c r="P38" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q38" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R38" s="16">
+        <v>0</v>
+      </c>
+      <c r="S38" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T38" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U38" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V38" s="16">
+        <v>1</v>
+      </c>
+      <c r="W38" s="16">
+        <v>1</v>
+      </c>
+      <c r="X38" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y38" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z38" s="16">
         <v>21</v>
       </c>
+      <c r="AB38" s="31">
+        <v>0</v>
+      </c>
     </row>
-    <row r="39" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D39" s="26" t="s">
+    <row r="39" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D39" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="E39" s="26">
+      <c r="E39" s="16">
         <v>1010011</v>
       </c>
-      <c r="F39" s="26">
-        <v>0</v>
-      </c>
-      <c r="G39" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H39" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I39" s="26">
-        <v>0</v>
-      </c>
-      <c r="J39" s="27" t="s">
+      <c r="F39" s="16">
+        <v>0</v>
+      </c>
+      <c r="G39" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H39" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I39" s="16">
+        <v>0</v>
+      </c>
+      <c r="J39" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K39" s="26">
-        <v>0</v>
-      </c>
-      <c r="L39" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M39" s="26">
-        <v>0</v>
-      </c>
-      <c r="N39" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O39" s="26">
+      <c r="K39" s="16">
+        <v>0</v>
+      </c>
+      <c r="L39" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M39" s="16">
+        <v>0</v>
+      </c>
+      <c r="N39" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O39" s="16">
         <v>10</v>
       </c>
-      <c r="P39" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q39" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R39" s="26">
-        <v>0</v>
-      </c>
-      <c r="S39" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T39" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U39" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V39" s="26">
-        <v>1</v>
-      </c>
-      <c r="W39" s="26">
-        <v>1</v>
-      </c>
-      <c r="X39" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y39" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z39" s="26">
+      <c r="P39" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q39" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R39" s="16">
+        <v>0</v>
+      </c>
+      <c r="S39" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T39" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U39" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V39" s="16">
+        <v>1</v>
+      </c>
+      <c r="W39" s="16">
+        <v>1</v>
+      </c>
+      <c r="X39" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y39" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z39" s="16">
         <v>18</v>
       </c>
+      <c r="AB39" s="30">
+        <v>1</v>
+      </c>
     </row>
-    <row r="40" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D40" s="26" t="s">
+    <row r="40" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D40" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="E40" s="26">
+      <c r="E40" s="16">
         <v>1010011</v>
       </c>
-      <c r="F40" s="26">
-        <v>0</v>
-      </c>
-      <c r="G40" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H40" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I40" s="26">
-        <v>0</v>
-      </c>
-      <c r="J40" s="27" t="s">
+      <c r="F40" s="16">
+        <v>0</v>
+      </c>
+      <c r="G40" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H40" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I40" s="16">
+        <v>0</v>
+      </c>
+      <c r="J40" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K40" s="26">
-        <v>0</v>
-      </c>
-      <c r="L40" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M40" s="26">
-        <v>0</v>
-      </c>
-      <c r="N40" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O40" s="26">
+      <c r="K40" s="16">
+        <v>0</v>
+      </c>
+      <c r="L40" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M40" s="16">
+        <v>0</v>
+      </c>
+      <c r="N40" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O40" s="16">
         <v>10</v>
       </c>
-      <c r="P40" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q40" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R40" s="26">
-        <v>0</v>
-      </c>
-      <c r="S40" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T40" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U40" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V40" s="26">
-        <v>1</v>
-      </c>
-      <c r="W40" s="26">
-        <v>1</v>
-      </c>
-      <c r="X40" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y40" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z40" s="26">
+      <c r="P40" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q40" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R40" s="16">
+        <v>0</v>
+      </c>
+      <c r="S40" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T40" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U40" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V40" s="16">
+        <v>1</v>
+      </c>
+      <c r="W40" s="16">
+        <v>1</v>
+      </c>
+      <c r="X40" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y40" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z40" s="16">
         <v>19</v>
       </c>
+      <c r="AB40" s="30">
+        <v>2</v>
+      </c>
     </row>
-    <row r="41" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D41" s="26" t="s">
+    <row r="41" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D41" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="E41" s="26">
+      <c r="E41" s="16">
         <v>1010011</v>
       </c>
-      <c r="F41" s="26">
-        <v>0</v>
-      </c>
-      <c r="G41" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H41" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I41" s="26">
-        <v>0</v>
-      </c>
-      <c r="J41" s="27" t="s">
+      <c r="F41" s="16">
+        <v>0</v>
+      </c>
+      <c r="G41" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H41" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I41" s="16">
+        <v>0</v>
+      </c>
+      <c r="J41" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K41" s="26">
-        <v>0</v>
-      </c>
-      <c r="L41" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M41" s="26">
-        <v>0</v>
-      </c>
-      <c r="N41" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O41" s="26">
+      <c r="K41" s="16">
+        <v>0</v>
+      </c>
+      <c r="L41" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M41" s="16">
+        <v>0</v>
+      </c>
+      <c r="N41" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O41" s="16">
         <v>10</v>
       </c>
-      <c r="P41" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q41" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R41" s="26">
-        <v>0</v>
-      </c>
-      <c r="S41" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T41" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U41" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V41" s="26">
-        <v>1</v>
-      </c>
-      <c r="W41" s="26">
-        <v>1</v>
-      </c>
-      <c r="X41" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y41" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z41" s="26">
+      <c r="P41" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q41" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R41" s="16">
+        <v>0</v>
+      </c>
+      <c r="S41" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T41" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U41" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V41" s="16">
+        <v>1</v>
+      </c>
+      <c r="W41" s="16">
+        <v>1</v>
+      </c>
+      <c r="X41" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y41" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z41" s="16">
         <v>20</v>
       </c>
+      <c r="AB41" s="30">
+        <v>3</v>
+      </c>
     </row>
-    <row r="42" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D42" s="26" t="s">
+    <row r="42" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D42" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="E42" s="26">
+      <c r="E42" s="16">
         <v>1010011</v>
       </c>
-      <c r="F42" s="26">
-        <v>0</v>
-      </c>
-      <c r="G42" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H42" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I42" s="26">
-        <v>0</v>
-      </c>
-      <c r="J42" s="27" t="s">
+      <c r="F42" s="16">
+        <v>0</v>
+      </c>
+      <c r="G42" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H42" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I42" s="16">
+        <v>0</v>
+      </c>
+      <c r="J42" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K42" s="26">
-        <v>0</v>
-      </c>
-      <c r="L42" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M42" s="26">
-        <v>0</v>
-      </c>
-      <c r="N42" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O42" s="26">
+      <c r="K42" s="16">
+        <v>0</v>
+      </c>
+      <c r="L42" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M42" s="16">
+        <v>0</v>
+      </c>
+      <c r="N42" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O42" s="16">
         <v>10</v>
       </c>
-      <c r="P42" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q42" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R42" s="26">
-        <v>0</v>
-      </c>
-      <c r="S42" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T42" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U42" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V42" s="26">
-        <v>1</v>
-      </c>
-      <c r="W42" s="26">
-        <v>1</v>
-      </c>
-      <c r="X42" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y42" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z42" s="26">
-        <v>16</v>
+      <c r="P42" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q42" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R42" s="16">
+        <v>0</v>
+      </c>
+      <c r="S42" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T42" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U42" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V42" s="16">
+        <v>1</v>
+      </c>
+      <c r="W42" s="16">
+        <v>1</v>
+      </c>
+      <c r="X42" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y42" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z42" s="16">
+        <v>16</v>
+      </c>
+      <c r="AB42" s="32">
+        <v>4</v>
       </c>
     </row>
-    <row r="43" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D43" s="26" t="s">
+    <row r="43" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D43" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="E43" s="26">
+      <c r="E43" s="16">
         <v>1010011</v>
       </c>
-      <c r="F43" s="26">
-        <v>0</v>
-      </c>
-      <c r="G43" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H43" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I43" s="26">
-        <v>0</v>
-      </c>
-      <c r="J43" s="27" t="s">
+      <c r="F43" s="16">
+        <v>0</v>
+      </c>
+      <c r="G43" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H43" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I43" s="16">
+        <v>0</v>
+      </c>
+      <c r="J43" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K43" s="26">
-        <v>0</v>
-      </c>
-      <c r="L43" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M43" s="26">
-        <v>0</v>
-      </c>
-      <c r="N43" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O43" s="26">
+      <c r="K43" s="16">
+        <v>0</v>
+      </c>
+      <c r="L43" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M43" s="16">
+        <v>0</v>
+      </c>
+      <c r="N43" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O43" s="16">
         <v>10</v>
       </c>
-      <c r="P43" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q43" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R43" s="26">
-        <v>0</v>
-      </c>
-      <c r="S43" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T43" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U43" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V43" s="26">
-        <v>1</v>
-      </c>
-      <c r="W43" s="26">
-        <v>1</v>
-      </c>
-      <c r="X43" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y43" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z43" s="26">
-        <v>15</v>
+      <c r="P43" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q43" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R43" s="16">
+        <v>0</v>
+      </c>
+      <c r="S43" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T43" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U43" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V43" s="16">
+        <v>1</v>
+      </c>
+      <c r="W43" s="16">
+        <v>1</v>
+      </c>
+      <c r="X43" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y43" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z43" s="16">
+        <v>15</v>
+      </c>
+      <c r="AB43" s="32">
+        <v>5</v>
       </c>
     </row>
-    <row r="44" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D44" s="26" t="s">
+    <row r="44" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D44" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="E44" s="26">
+      <c r="E44" s="16">
         <v>1010011</v>
       </c>
-      <c r="F44" s="26">
-        <v>0</v>
-      </c>
-      <c r="G44" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H44" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I44" s="26">
-        <v>0</v>
-      </c>
-      <c r="J44" s="27" t="s">
+      <c r="F44" s="16">
+        <v>0</v>
+      </c>
+      <c r="G44" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H44" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I44" s="16">
+        <v>0</v>
+      </c>
+      <c r="J44" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K44" s="26">
-        <v>0</v>
-      </c>
-      <c r="L44" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M44" s="26">
-        <v>0</v>
-      </c>
-      <c r="N44" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O44" s="26">
+      <c r="K44" s="16">
+        <v>0</v>
+      </c>
+      <c r="L44" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M44" s="16">
+        <v>0</v>
+      </c>
+      <c r="N44" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O44" s="16">
         <v>10</v>
       </c>
-      <c r="P44" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q44" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R44" s="26">
-        <v>0</v>
-      </c>
-      <c r="S44" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T44" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U44" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V44" s="26">
-        <v>1</v>
-      </c>
-      <c r="W44" s="26">
-        <v>1</v>
-      </c>
-      <c r="X44" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y44" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z44" s="26">
+      <c r="P44" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q44" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R44" s="16">
+        <v>0</v>
+      </c>
+      <c r="S44" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T44" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U44" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V44" s="16">
+        <v>1</v>
+      </c>
+      <c r="W44" s="16">
+        <v>1</v>
+      </c>
+      <c r="X44" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y44" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z44" s="16">
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D45" s="26" t="s">
+    <row r="45" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D45" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="E45" s="26">
+      <c r="E45" s="16">
         <v>1010011</v>
       </c>
-      <c r="F45" s="26">
-        <v>0</v>
-      </c>
-      <c r="G45" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H45" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I45" s="26">
-        <v>0</v>
-      </c>
-      <c r="J45" s="27" t="s">
+      <c r="F45" s="16">
+        <v>0</v>
+      </c>
+      <c r="G45" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H45" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I45" s="16">
+        <v>0</v>
+      </c>
+      <c r="J45" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K45" s="26">
-        <v>0</v>
-      </c>
-      <c r="L45" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M45" s="26">
-        <v>0</v>
-      </c>
-      <c r="N45" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O45" s="26">
+      <c r="K45" s="16">
+        <v>0</v>
+      </c>
+      <c r="L45" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M45" s="16">
+        <v>0</v>
+      </c>
+      <c r="N45" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O45" s="16">
         <v>10</v>
       </c>
-      <c r="P45" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q45" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R45" s="26">
-        <v>0</v>
-      </c>
-      <c r="S45" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T45" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U45" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V45" s="26">
-        <v>1</v>
-      </c>
-      <c r="W45" s="26">
-        <v>1</v>
-      </c>
-      <c r="X45" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y45" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z45" s="26">
+      <c r="P45" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q45" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R45" s="16">
+        <v>0</v>
+      </c>
+      <c r="S45" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T45" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U45" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V45" s="16">
+        <v>1</v>
+      </c>
+      <c r="W45" s="16">
+        <v>1</v>
+      </c>
+      <c r="X45" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y45" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z45" s="16">
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D46" s="26" t="s">
+    <row r="46" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D46" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="E46" s="26">
+      <c r="E46" s="16">
         <v>1010011</v>
       </c>
-      <c r="F46" s="26">
-        <v>0</v>
-      </c>
-      <c r="G46" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H46" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I46" s="26">
-        <v>0</v>
-      </c>
-      <c r="J46" s="27" t="s">
+      <c r="F46" s="16">
+        <v>0</v>
+      </c>
+      <c r="G46" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H46" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I46" s="16">
+        <v>0</v>
+      </c>
+      <c r="J46" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K46" s="26">
-        <v>0</v>
-      </c>
-      <c r="L46" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M46" s="26">
-        <v>0</v>
-      </c>
-      <c r="N46" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O46" s="26">
+      <c r="K46" s="16">
+        <v>0</v>
+      </c>
+      <c r="L46" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M46" s="16">
+        <v>0</v>
+      </c>
+      <c r="N46" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O46" s="16">
         <v>10</v>
       </c>
-      <c r="P46" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q46" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R46" s="26">
-        <v>0</v>
-      </c>
-      <c r="S46" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T46" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U46" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V46" s="26">
-        <v>1</v>
-      </c>
-      <c r="W46" s="26">
-        <v>1</v>
-      </c>
-      <c r="X46" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y46" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z46" s="26">
+      <c r="P46" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q46" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R46" s="16">
+        <v>0</v>
+      </c>
+      <c r="S46" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T46" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U46" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V46" s="16">
+        <v>1</v>
+      </c>
+      <c r="W46" s="16">
+        <v>1</v>
+      </c>
+      <c r="X46" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y46" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z46" s="16">
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D47" s="26" t="s">
+    <row r="47" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D47" s="16" t="s">
         <v>111</v>
       </c>
-      <c r="E47" s="26">
+      <c r="E47" s="16">
         <v>1010011</v>
       </c>
-      <c r="F47" s="26">
-        <v>0</v>
-      </c>
-      <c r="G47" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H47" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I47" s="26">
-        <v>0</v>
-      </c>
-      <c r="J47" s="27" t="s">
+      <c r="F47" s="16">
+        <v>0</v>
+      </c>
+      <c r="G47" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H47" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I47" s="16">
+        <v>0</v>
+      </c>
+      <c r="J47" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K47" s="26">
-        <v>0</v>
-      </c>
-      <c r="L47" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M47" s="26">
-        <v>0</v>
-      </c>
-      <c r="N47" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O47" s="26">
+      <c r="K47" s="16">
+        <v>0</v>
+      </c>
+      <c r="L47" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M47" s="16">
+        <v>0</v>
+      </c>
+      <c r="N47" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O47" s="16">
         <v>10</v>
       </c>
-      <c r="P47" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q47" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R47" s="26">
-        <v>0</v>
-      </c>
-      <c r="S47" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T47" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U47" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V47" s="26">
-        <v>1</v>
-      </c>
-      <c r="W47" s="26">
-        <v>1</v>
-      </c>
-      <c r="X47" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y47" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z47" s="26">
+      <c r="P47" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q47" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R47" s="16">
+        <v>0</v>
+      </c>
+      <c r="S47" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T47" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U47" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V47" s="16">
+        <v>1</v>
+      </c>
+      <c r="W47" s="16">
+        <v>1</v>
+      </c>
+      <c r="X47" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y47" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z47" s="16">
         <v>6</v>
       </c>
     </row>
-    <row r="48" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D48" s="26" t="s">
+    <row r="48" spans="4:28" x14ac:dyDescent="0.3">
+      <c r="D48" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="E48" s="26">
+      <c r="E48" s="16">
         <v>1010011</v>
       </c>
-      <c r="F48" s="26">
-        <v>1</v>
-      </c>
-      <c r="G48" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H48" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I48" s="26">
-        <v>0</v>
-      </c>
-      <c r="J48" s="27" t="s">
+      <c r="F48" s="16">
+        <v>1</v>
+      </c>
+      <c r="G48" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H48" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I48" s="16">
+        <v>0</v>
+      </c>
+      <c r="J48" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K48" s="26">
-        <v>0</v>
-      </c>
-      <c r="L48" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M48" s="26">
-        <v>0</v>
-      </c>
-      <c r="N48" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O48" s="26">
+      <c r="K48" s="16">
+        <v>0</v>
+      </c>
+      <c r="L48" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M48" s="16">
+        <v>0</v>
+      </c>
+      <c r="N48" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O48" s="16">
         <v>10</v>
       </c>
-      <c r="P48" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q48" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R48" s="26">
-        <v>0</v>
-      </c>
-      <c r="S48" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T48" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U48" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V48" s="26">
-        <v>0</v>
-      </c>
-      <c r="W48" s="26">
-        <v>1</v>
-      </c>
-      <c r="X48" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y48" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z48" s="26">
+      <c r="P48" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q48" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R48" s="16">
+        <v>0</v>
+      </c>
+      <c r="S48" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T48" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U48" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V48" s="16">
+        <v>0</v>
+      </c>
+      <c r="W48" s="16">
+        <v>1</v>
+      </c>
+      <c r="X48" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y48" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z48" s="16">
         <v>22</v>
       </c>
     </row>
     <row r="49" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D49" s="26" t="s">
+      <c r="D49" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="E49" s="26">
+      <c r="E49" s="16">
         <v>1010011</v>
       </c>
-      <c r="F49" s="26">
-        <v>0</v>
-      </c>
-      <c r="G49" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H49" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I49" s="26">
-        <v>0</v>
-      </c>
-      <c r="J49" s="27" t="s">
+      <c r="F49" s="16">
+        <v>0</v>
+      </c>
+      <c r="G49" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H49" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I49" s="16">
+        <v>0</v>
+      </c>
+      <c r="J49" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K49" s="26">
-        <v>0</v>
-      </c>
-      <c r="L49" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M49" s="26">
-        <v>0</v>
-      </c>
-      <c r="N49" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O49" s="26">
+      <c r="K49" s="16">
+        <v>0</v>
+      </c>
+      <c r="L49" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M49" s="16">
+        <v>0</v>
+      </c>
+      <c r="N49" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O49" s="16">
         <v>10</v>
       </c>
-      <c r="P49" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q49" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R49" s="26">
-        <v>0</v>
-      </c>
-      <c r="S49" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T49" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U49" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V49" s="26">
-        <v>1</v>
-      </c>
-      <c r="W49" s="26">
-        <v>1</v>
-      </c>
-      <c r="X49" s="26">
-        <v>0</v>
-      </c>
-      <c r="Y49" s="26">
-        <v>0</v>
-      </c>
-      <c r="Z49" s="26">
+      <c r="P49" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q49" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R49" s="16">
+        <v>0</v>
+      </c>
+      <c r="S49" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T49" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U49" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V49" s="16">
+        <v>1</v>
+      </c>
+      <c r="W49" s="16">
+        <v>1</v>
+      </c>
+      <c r="X49" s="16">
+        <v>0</v>
+      </c>
+      <c r="Y49" s="16">
+        <v>0</v>
+      </c>
+      <c r="Z49" s="16">
         <v>22</v>
       </c>
     </row>
     <row r="50" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D50" s="26" t="s">
+      <c r="D50" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="E50" s="26">
+      <c r="E50" s="16">
         <v>1010011</v>
       </c>
-      <c r="F50" s="26">
-        <v>0</v>
-      </c>
-      <c r="G50" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H50" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I50" s="26">
-        <v>0</v>
-      </c>
-      <c r="J50" s="27" t="s">
+      <c r="F50" s="16">
+        <v>0</v>
+      </c>
+      <c r="G50" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H50" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I50" s="16">
+        <v>0</v>
+      </c>
+      <c r="J50" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K50" s="26">
-        <v>0</v>
-      </c>
-      <c r="L50" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M50" s="26">
-        <v>0</v>
-      </c>
-      <c r="N50" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O50" s="26">
+      <c r="K50" s="16">
+        <v>0</v>
+      </c>
+      <c r="L50" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M50" s="16">
+        <v>0</v>
+      </c>
+      <c r="N50" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O50" s="16">
         <v>10</v>
       </c>
-      <c r="P50" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q50" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R50" s="26">
-        <v>0</v>
-      </c>
-      <c r="S50" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T50" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U50" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V50" s="26">
-        <v>1</v>
-      </c>
-      <c r="W50" s="26">
-        <v>1</v>
-      </c>
-      <c r="X50" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y50" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z50" s="26">
+      <c r="P50" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q50" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R50" s="16">
+        <v>0</v>
+      </c>
+      <c r="S50" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T50" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U50" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V50" s="16">
+        <v>1</v>
+      </c>
+      <c r="W50" s="16">
+        <v>1</v>
+      </c>
+      <c r="X50" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y50" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z50" s="16">
         <v>8</v>
       </c>
     </row>
     <row r="51" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D51" s="26" t="s">
+      <c r="D51" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="E51" s="26">
+      <c r="E51" s="16">
         <v>1010011</v>
       </c>
-      <c r="F51" s="26">
-        <v>0</v>
-      </c>
-      <c r="G51" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H51" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I51" s="26">
-        <v>0</v>
-      </c>
-      <c r="J51" s="27" t="s">
+      <c r="F51" s="16">
+        <v>0</v>
+      </c>
+      <c r="G51" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H51" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I51" s="16">
+        <v>0</v>
+      </c>
+      <c r="J51" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K51" s="26">
-        <v>0</v>
-      </c>
-      <c r="L51" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M51" s="26">
-        <v>0</v>
-      </c>
-      <c r="N51" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O51" s="26">
+      <c r="K51" s="16">
+        <v>0</v>
+      </c>
+      <c r="L51" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M51" s="16">
+        <v>0</v>
+      </c>
+      <c r="N51" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O51" s="16">
         <v>10</v>
       </c>
-      <c r="P51" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q51" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R51" s="26">
-        <v>0</v>
-      </c>
-      <c r="S51" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T51" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U51" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V51" s="26">
-        <v>1</v>
-      </c>
-      <c r="W51" s="26">
-        <v>1</v>
-      </c>
-      <c r="X51" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y51" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z51" s="26">
+      <c r="P51" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q51" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R51" s="16">
+        <v>0</v>
+      </c>
+      <c r="S51" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T51" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U51" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V51" s="16">
+        <v>1</v>
+      </c>
+      <c r="W51" s="16">
+        <v>1</v>
+      </c>
+      <c r="X51" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y51" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z51" s="16">
         <v>10</v>
       </c>
     </row>
     <row r="52" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D52" s="26" t="s">
+      <c r="D52" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="E52" s="26">
+      <c r="E52" s="16">
         <v>1010011</v>
       </c>
-      <c r="F52" s="26">
-        <v>0</v>
-      </c>
-      <c r="G52" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H52" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I52" s="26">
-        <v>0</v>
-      </c>
-      <c r="J52" s="27" t="s">
+      <c r="F52" s="16">
+        <v>0</v>
+      </c>
+      <c r="G52" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H52" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I52" s="16">
+        <v>0</v>
+      </c>
+      <c r="J52" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K52" s="26">
-        <v>0</v>
-      </c>
-      <c r="L52" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M52" s="26">
-        <v>0</v>
-      </c>
-      <c r="N52" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O52" s="26">
+      <c r="K52" s="16">
+        <v>0</v>
+      </c>
+      <c r="L52" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M52" s="16">
+        <v>0</v>
+      </c>
+      <c r="N52" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O52" s="16">
         <v>10</v>
       </c>
-      <c r="P52" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q52" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R52" s="26">
-        <v>0</v>
-      </c>
-      <c r="S52" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T52" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U52" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V52" s="26">
-        <v>1</v>
-      </c>
-      <c r="W52" s="26">
-        <v>1</v>
-      </c>
-      <c r="X52" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y52" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z52" s="26">
+      <c r="P52" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q52" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R52" s="16">
+        <v>0</v>
+      </c>
+      <c r="S52" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T52" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U52" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V52" s="16">
+        <v>1</v>
+      </c>
+      <c r="W52" s="16">
+        <v>1</v>
+      </c>
+      <c r="X52" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y52" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z52" s="16">
         <v>9</v>
       </c>
     </row>
     <row r="53" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D53" s="26" t="s">
+      <c r="D53" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="E53" s="26">
+      <c r="E53" s="16">
         <v>1010011</v>
       </c>
-      <c r="F53" s="26">
-        <v>0</v>
-      </c>
-      <c r="G53" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="H53" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I53" s="26">
-        <v>0</v>
-      </c>
-      <c r="J53" s="27" t="s">
+      <c r="F53" s="16">
+        <v>0</v>
+      </c>
+      <c r="G53" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H53" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I53" s="16">
+        <v>0</v>
+      </c>
+      <c r="J53" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K53" s="26">
-        <v>0</v>
-      </c>
-      <c r="L53" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M53" s="26">
-        <v>0</v>
-      </c>
-      <c r="N53" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="O53" s="26">
+      <c r="K53" s="16">
+        <v>0</v>
+      </c>
+      <c r="L53" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="M53" s="16">
+        <v>0</v>
+      </c>
+      <c r="N53" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="O53" s="16">
         <v>10</v>
       </c>
-      <c r="P53" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q53" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="R53" s="26">
-        <v>0</v>
-      </c>
-      <c r="S53" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="T53" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="U53" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="V53" s="26">
-        <v>1</v>
-      </c>
-      <c r="W53" s="26">
-        <v>1</v>
-      </c>
-      <c r="X53" s="26">
-        <v>1</v>
-      </c>
-      <c r="Y53" s="26">
-        <v>1</v>
-      </c>
-      <c r="Z53" s="26">
+      <c r="P53" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q53" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="R53" s="16">
+        <v>0</v>
+      </c>
+      <c r="S53" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="T53" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="U53" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="V53" s="16">
+        <v>1</v>
+      </c>
+      <c r="W53" s="16">
+        <v>1</v>
+      </c>
+      <c r="X53" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y53" s="16">
+        <v>1</v>
+      </c>
+      <c r="Z53" s="16">
         <v>2</v>
       </c>
     </row>
@@ -5260,20 +5306,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="aa762089-36ad-4bf7-9314-c7223c4b604d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="aa762089-36ad-4bf7-9314-c7223c4b604d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5295,14 +5341,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A7B8669E-67F1-4457-BB68-A16754986870}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E0D4C47-9B8A-40A7-B507-77A4C6E21046}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -5316,4 +5354,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A7B8669E-67F1-4457-BB68-A16754986870}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update for forwading F, M, I, have bug in fsw and flw
</commit_message>
<xml_diff>
--- a/Control.xlsx
+++ b/Control.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Hung\Khoa_Luan\ISS-RV32ICMFA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A3298FA-14F9-4BCE-BAF9-344F73BED60E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{209292B6-A009-4256-A7D4-680CE3A45562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CF86E8A2-CD57-4282-A2FF-4C2B018B82AC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="137">
   <si>
     <t>instructions</t>
   </si>
@@ -717,6 +717,15 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -745,15 +754,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1090,9 +1090,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{690C58A5-C37A-4C5A-8C40-61E7ED87ACAD}">
-  <dimension ref="D3:AO54"/>
+  <dimension ref="A3:AO54"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="3" max="3" width="8.88671875" customWidth="1"/>
     <col min="4" max="4" width="12.77734375" customWidth="1"/>
     <col min="14" max="16" width="16.33203125" customWidth="1"/>
     <col min="17" max="17" width="18.109375" customWidth="1"/>
@@ -1111,31 +1112,31 @@
   </cols>
   <sheetData>
     <row r="3" spans="4:41" x14ac:dyDescent="0.3">
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="21"/>
-      <c r="O3" s="21"/>
-      <c r="P3" s="21"/>
-      <c r="Q3" s="21"/>
-      <c r="R3" s="21"/>
-      <c r="S3" s="21"/>
-      <c r="T3" s="21"/>
-      <c r="U3" s="21"/>
-      <c r="V3" s="21"/>
-      <c r="W3" s="21"/>
-      <c r="X3" s="21"/>
-      <c r="Y3" s="21"/>
-      <c r="Z3" s="22"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="24"/>
+      <c r="L3" s="24"/>
+      <c r="M3" s="24"/>
+      <c r="N3" s="24"/>
+      <c r="O3" s="24"/>
+      <c r="P3" s="24"/>
+      <c r="Q3" s="24"/>
+      <c r="R3" s="24"/>
+      <c r="S3" s="24"/>
+      <c r="T3" s="24"/>
+      <c r="U3" s="24"/>
+      <c r="V3" s="24"/>
+      <c r="W3" s="24"/>
+      <c r="X3" s="24"/>
+      <c r="Y3" s="24"/>
+      <c r="Z3" s="25"/>
       <c r="AB3" t="s">
         <v>17</v>
       </c>
@@ -1468,7 +1469,7 @@
       <c r="Z7" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="AB7" s="23">
+      <c r="AB7" s="26">
         <v>10</v>
       </c>
       <c r="AC7" s="2" t="s">
@@ -1554,7 +1555,7 @@
       <c r="Z8" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="AB8" s="24"/>
+      <c r="AB8" s="27"/>
       <c r="AC8" s="2" t="s">
         <v>25</v>
       </c>
@@ -1638,7 +1639,7 @@
       <c r="Z9" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="AB9" s="24"/>
+      <c r="AB9" s="27"/>
       <c r="AC9" s="2" t="s">
         <v>26</v>
       </c>
@@ -1657,12 +1658,12 @@
       <c r="AI9" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="AJ9" s="27" t="s">
+      <c r="AJ9" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="AK9" s="27"/>
-      <c r="AL9" s="27"/>
-      <c r="AM9" s="27"/>
+      <c r="AK9" s="30"/>
+      <c r="AL9" s="30"/>
+      <c r="AM9" s="30"/>
       <c r="AN9" s="1" t="s">
         <v>75</v>
       </c>
@@ -1740,7 +1741,7 @@
       <c r="Z10" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="AB10" s="24"/>
+      <c r="AB10" s="27"/>
       <c r="AC10" s="1">
         <v>110</v>
       </c>
@@ -1842,7 +1843,7 @@
       <c r="Z11" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="AB11" s="25"/>
+      <c r="AB11" s="28"/>
       <c r="AC11" s="1">
         <v>111</v>
       </c>
@@ -2642,17 +2643,17 @@
       <c r="AH22" t="s">
         <v>77</v>
       </c>
-      <c r="AI22" s="28" t="s">
+      <c r="AI22" s="31" t="s">
         <v>81</v>
       </c>
-      <c r="AJ22" s="28"/>
-      <c r="AK22" s="28"/>
-      <c r="AL22" s="28" t="s">
+      <c r="AJ22" s="31"/>
+      <c r="AK22" s="31"/>
+      <c r="AL22" s="31" t="s">
         <v>82</v>
       </c>
-      <c r="AM22" s="28"/>
-      <c r="AN22" s="28"/>
-      <c r="AO22" s="28"/>
+      <c r="AM22" s="31"/>
+      <c r="AN22" s="31"/>
+      <c r="AO22" s="31"/>
     </row>
     <row r="23" spans="4:41" x14ac:dyDescent="0.3">
       <c r="D23" s="11" t="s">
@@ -2742,17 +2743,17 @@
       <c r="AH23" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="AI23" s="27" t="s">
+      <c r="AI23" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="AJ23" s="27"/>
-      <c r="AK23" s="27"/>
-      <c r="AL23" s="27" t="s">
+      <c r="AJ23" s="30"/>
+      <c r="AK23" s="30"/>
+      <c r="AL23" s="30" t="s">
         <v>80</v>
       </c>
-      <c r="AM23" s="27"/>
-      <c r="AN23" s="27"/>
-      <c r="AO23" s="27"/>
+      <c r="AM23" s="30"/>
+      <c r="AN23" s="30"/>
+      <c r="AO23" s="30"/>
     </row>
     <row r="24" spans="4:41" x14ac:dyDescent="0.3">
       <c r="D24" s="11" t="s">
@@ -2910,7 +2911,7 @@
       <c r="Z25" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="AB25" s="26">
+      <c r="AB25" s="29">
         <v>1</v>
       </c>
       <c r="AC25" s="1">
@@ -2932,12 +2933,12 @@
         <v>84</v>
       </c>
       <c r="AJ25" s="3"/>
-      <c r="AK25" s="29" t="s">
+      <c r="AK25" s="32" t="s">
         <v>85</v>
       </c>
-      <c r="AL25" s="29"/>
-      <c r="AM25" s="29"/>
-      <c r="AN25" s="29"/>
+      <c r="AL25" s="32"/>
+      <c r="AM25" s="32"/>
+      <c r="AN25" s="32"/>
     </row>
     <row r="26" spans="4:41" x14ac:dyDescent="0.3">
       <c r="D26" s="15" t="s">
@@ -3009,7 +3010,7 @@
       <c r="Z26" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="AB26" s="26"/>
+      <c r="AB26" s="29"/>
       <c r="AC26" s="2">
         <v>1</v>
       </c>
@@ -3025,16 +3026,16 @@
       <c r="AH26" s="3">
         <v>0</v>
       </c>
-      <c r="AI26" s="29">
+      <c r="AI26" s="32">
         <v>-127</v>
       </c>
-      <c r="AJ26" s="29"/>
-      <c r="AK26" s="29" t="s">
+      <c r="AJ26" s="32"/>
+      <c r="AK26" s="32" t="s">
         <v>88</v>
       </c>
-      <c r="AL26" s="29"/>
-      <c r="AM26" s="29"/>
-      <c r="AN26" s="29"/>
+      <c r="AL26" s="32"/>
+      <c r="AM26" s="32"/>
+      <c r="AN26" s="32"/>
     </row>
     <row r="27" spans="4:41" x14ac:dyDescent="0.3">
       <c r="D27" s="15" t="s">
@@ -3106,7 +3107,7 @@
       <c r="Z27" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="AB27" s="26"/>
+      <c r="AB27" s="29"/>
       <c r="AC27" s="2">
         <v>2</v>
       </c>
@@ -3122,16 +3123,16 @@
       <c r="AH27" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="AI27" s="26" t="s">
+      <c r="AI27" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="AJ27" s="26"/>
-      <c r="AK27" s="29" t="s">
+      <c r="AJ27" s="29"/>
+      <c r="AK27" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="AL27" s="29"/>
-      <c r="AM27" s="29"/>
-      <c r="AN27" s="29"/>
+      <c r="AL27" s="32"/>
+      <c r="AM27" s="32"/>
+      <c r="AN27" s="32"/>
     </row>
     <row r="28" spans="4:41" x14ac:dyDescent="0.3">
       <c r="D28" s="16" t="s">
@@ -3203,7 +3204,7 @@
       <c r="Z28" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="AB28" s="26"/>
+      <c r="AB28" s="29"/>
       <c r="AC28" s="2">
         <v>3</v>
       </c>
@@ -3219,16 +3220,16 @@
       <c r="AH28" s="3">
         <v>255</v>
       </c>
-      <c r="AI28" s="29">
+      <c r="AI28" s="32">
         <v>128</v>
       </c>
-      <c r="AJ28" s="29"/>
-      <c r="AK28" s="29" t="s">
+      <c r="AJ28" s="32"/>
+      <c r="AK28" s="32" t="s">
         <v>90</v>
       </c>
-      <c r="AL28" s="29"/>
-      <c r="AM28" s="29"/>
-      <c r="AN28" s="29"/>
+      <c r="AL28" s="32"/>
+      <c r="AM28" s="32"/>
+      <c r="AN28" s="32"/>
     </row>
     <row r="29" spans="4:41" x14ac:dyDescent="0.3">
       <c r="D29" s="16" t="s">
@@ -3300,7 +3301,7 @@
       <c r="Z29" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="AB29" s="26"/>
+      <c r="AB29" s="29"/>
       <c r="AC29" s="1">
         <v>4</v>
       </c>
@@ -3384,7 +3385,7 @@
       <c r="Z30" s="18">
         <v>11</v>
       </c>
-      <c r="AB30" s="26"/>
+      <c r="AB30" s="29"/>
       <c r="AC30" s="1">
         <v>5</v>
       </c>
@@ -3468,7 +3469,7 @@
       <c r="Z31" s="18">
         <v>12</v>
       </c>
-      <c r="AB31" s="26"/>
+      <c r="AB31" s="29"/>
       <c r="AC31" s="1">
         <v>6</v>
       </c>
@@ -3552,7 +3553,7 @@
       <c r="Z32" s="18">
         <v>13</v>
       </c>
-      <c r="AB32" s="26"/>
+      <c r="AB32" s="29"/>
       <c r="AC32" s="1">
         <v>7</v>
       </c>
@@ -3994,7 +3995,7 @@
       <c r="Z38" s="16">
         <v>21</v>
       </c>
-      <c r="AB38" s="31">
+      <c r="AB38" s="21">
         <v>0</v>
       </c>
     </row>
@@ -4068,7 +4069,7 @@
       <c r="Z39" s="16">
         <v>18</v>
       </c>
-      <c r="AB39" s="30">
+      <c r="AB39" s="20">
         <v>1</v>
       </c>
     </row>
@@ -4142,7 +4143,7 @@
       <c r="Z40" s="16">
         <v>19</v>
       </c>
-      <c r="AB40" s="30">
+      <c r="AB40" s="20">
         <v>2</v>
       </c>
     </row>
@@ -4216,7 +4217,7 @@
       <c r="Z41" s="16">
         <v>20</v>
       </c>
-      <c r="AB41" s="30">
+      <c r="AB41" s="20">
         <v>3</v>
       </c>
     </row>
@@ -4290,7 +4291,7 @@
       <c r="Z42" s="16">
         <v>16</v>
       </c>
-      <c r="AB42" s="32">
+      <c r="AB42" s="22">
         <v>4</v>
       </c>
     </row>
@@ -4364,7 +4365,7 @@
       <c r="Z43" s="16">
         <v>15</v>
       </c>
-      <c r="AB43" s="32">
+      <c r="AB43" s="22">
         <v>5</v>
       </c>
     </row>
@@ -4430,10 +4431,10 @@
         <v>1</v>
       </c>
       <c r="X44" s="16">
-        <v>1</v>
-      </c>
-      <c r="Y44" s="16">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y44" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="Z44" s="16">
         <v>3</v>
@@ -4501,10 +4502,10 @@
         <v>1</v>
       </c>
       <c r="X45" s="16">
-        <v>1</v>
-      </c>
-      <c r="Y45" s="16">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y45" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="Z45" s="16">
         <v>4</v>
@@ -4518,7 +4519,7 @@
         <v>1010011</v>
       </c>
       <c r="F46" s="16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G46" s="16" t="s">
         <v>46</v>
@@ -4566,7 +4567,7 @@
         <v>46</v>
       </c>
       <c r="V46" s="16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W46" s="16">
         <v>1</v>
@@ -4574,8 +4575,8 @@
       <c r="X46" s="16">
         <v>1</v>
       </c>
-      <c r="Y46" s="16">
-        <v>1</v>
+      <c r="Y46" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="Z46" s="16">
         <v>5</v>
@@ -4589,7 +4590,7 @@
         <v>1010011</v>
       </c>
       <c r="F47" s="16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G47" s="16" t="s">
         <v>46</v>
@@ -4637,7 +4638,7 @@
         <v>46</v>
       </c>
       <c r="V47" s="16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W47" s="16">
         <v>1</v>
@@ -4645,8 +4646,8 @@
       <c r="X47" s="16">
         <v>1</v>
       </c>
-      <c r="Y47" s="16">
-        <v>1</v>
+      <c r="Y47" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="Z47" s="16">
         <v>6</v>
@@ -4716,14 +4717,14 @@
       <c r="X48" s="16">
         <v>1</v>
       </c>
-      <c r="Y48" s="16">
-        <v>1</v>
+      <c r="Y48" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="Z48" s="16">
         <v>22</v>
       </c>
     </row>
-    <row r="49" spans="4:26" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:26" x14ac:dyDescent="0.3">
       <c r="D49" s="16" t="s">
         <v>113</v>
       </c>
@@ -4787,14 +4788,14 @@
       <c r="X49" s="16">
         <v>0</v>
       </c>
-      <c r="Y49" s="16">
-        <v>0</v>
+      <c r="Y49" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="Z49" s="16">
         <v>22</v>
       </c>
     </row>
-    <row r="50" spans="4:26" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:26" x14ac:dyDescent="0.3">
       <c r="D50" s="16" t="s">
         <v>114</v>
       </c>
@@ -4865,7 +4866,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="4:26" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:26" x14ac:dyDescent="0.3">
       <c r="D51" s="16" t="s">
         <v>115</v>
       </c>
@@ -4936,7 +4937,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="52" spans="4:26" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:26" x14ac:dyDescent="0.3">
       <c r="D52" s="16" t="s">
         <v>116</v>
       </c>
@@ -5007,7 +5008,10 @@
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="4:26" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>16</v>
+      </c>
       <c r="D53" s="16" t="s">
         <v>117</v>
       </c>
@@ -5015,7 +5019,7 @@
         <v>1010011</v>
       </c>
       <c r="F53" s="16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G53" s="16" t="s">
         <v>46</v>
@@ -5063,7 +5067,7 @@
         <v>46</v>
       </c>
       <c r="V53" s="16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W53" s="16">
         <v>1</v>
@@ -5071,14 +5075,14 @@
       <c r="X53" s="16">
         <v>1</v>
       </c>
-      <c r="Y53" s="16">
-        <v>1</v>
+      <c r="Y53" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="Z53" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="4:26" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:26" x14ac:dyDescent="0.3">
       <c r="J54" s="4"/>
     </row>
   </sheetData>
@@ -5306,20 +5310,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="aa762089-36ad-4bf7-9314-c7223c4b604d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="aa762089-36ad-4bf7-9314-c7223c4b604d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5341,6 +5345,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A7B8669E-67F1-4457-BB68-A16754986870}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E0D4C47-9B8A-40A7-B507-77A4C6E21046}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -5354,12 +5366,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A7B8669E-67F1-4457-BB68-A16754986870}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>